<commit_message>
Corrected Resource manangement logic
</commit_message>
<xml_diff>
--- a/5.5.13 Real Property-Monthly Reviews-2_results.xlsx
+++ b/5.5.13 Real Property-Monthly Reviews-2_results.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>44.14</v>
+        <v>29.79</v>
       </c>
     </row>
     <row r="3">
@@ -464,7 +464,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.33</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
@@ -570,43 +570,43 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>500</v>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E2" t="n">
-        <v>100</v>
+        <v>19.6</v>
       </c>
       <c r="F2" t="n">
-        <v>55.67</v>
+        <v>105.69</v>
       </c>
       <c r="G2" t="n">
-        <v>1436.28</v>
+        <v>28924.26</v>
       </c>
       <c r="H2" t="n">
-        <v>247.94</v>
+        <v>16728.64</v>
       </c>
       <c r="I2" t="n">
-        <v>104.44</v>
+        <v>24395.45</v>
       </c>
       <c r="J2" t="n">
-        <v>400.58</v>
+        <v>10682.1</v>
       </c>
       <c r="K2" t="n">
-        <v>403.6</v>
+        <v>27274.05</v>
       </c>
       <c r="L2" t="n">
-        <v>675.17</v>
+        <v>1608681.15</v>
       </c>
       <c r="M2" t="n">
-        <v>30.07</v>
+        <v>78.54000000000001</v>
       </c>
       <c r="N2" t="n">
-        <v>91.56999999999999</v>
+        <v>28903.7</v>
       </c>
       <c r="O2" t="n">
-        <v>67.52</v>
+        <v>16415.11</v>
       </c>
     </row>
     <row r="3">
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10</v>
+        <v>500</v>
       </c>
       <c r="D3" t="n">
-        <v>10</v>
+        <v>500</v>
       </c>
       <c r="E3" t="n">
         <v>100</v>
@@ -672,43 +672,43 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>496</v>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>496</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>5.29</v>
+        <v>5.12</v>
       </c>
       <c r="G4" t="n">
-        <v>9.039999999999999</v>
+        <v>9.58</v>
       </c>
       <c r="H4" t="n">
-        <v>7.55</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>8.029999999999999</v>
+        <v>8.18</v>
       </c>
       <c r="J4" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="K4" t="n">
-        <v>8.82</v>
+        <v>9.34</v>
       </c>
       <c r="L4" t="n">
-        <v>520.1799999999999</v>
+        <v>12164872.29</v>
       </c>
       <c r="M4" t="n">
-        <v>6.21</v>
+        <v>5.71</v>
       </c>
       <c r="N4" t="n">
-        <v>54.33</v>
+        <v>21931.43</v>
       </c>
       <c r="O4" t="n">
-        <v>28.9</v>
+        <v>12238.3</v>
       </c>
     </row>
     <row r="5">
@@ -723,10 +723,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10</v>
+        <v>496</v>
       </c>
       <c r="D5" t="n">
-        <v>10</v>
+        <v>496</v>
       </c>
       <c r="E5" t="n">
         <v>100</v>
@@ -774,43 +774,43 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>76</v>
       </c>
       <c r="D6" t="n">
-        <v>9</v>
+        <v>76</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>4.29</v>
+        <v>3.4</v>
       </c>
       <c r="G6" t="n">
-        <v>6.57</v>
+        <v>6.71</v>
       </c>
       <c r="H6" t="n">
-        <v>5.35</v>
+        <v>5.46</v>
       </c>
       <c r="I6" t="n">
-        <v>5.21</v>
+        <v>5.49</v>
       </c>
       <c r="J6" t="n">
-        <v>0.75</v>
+        <v>0.92</v>
       </c>
       <c r="K6" t="n">
-        <v>6.35</v>
+        <v>6.58</v>
       </c>
       <c r="L6" t="n">
-        <v>1894.43</v>
+        <v>2459394.43</v>
       </c>
       <c r="M6" t="n">
-        <v>26.5</v>
+        <v>72.83</v>
       </c>
       <c r="N6" t="n">
-        <v>1150.06</v>
+        <v>25765.28</v>
       </c>
       <c r="O6" t="n">
-        <v>111.44</v>
+        <v>16287.38</v>
       </c>
     </row>
     <row r="7">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="D7" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E7" t="n">
         <v>100</v>
@@ -852,16 +852,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>9.32</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>9.32</v>
       </c>
       <c r="N7" t="n">
-        <v>0</v>
+        <v>9.32</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>9.32</v>
       </c>
     </row>
     <row r="8">
@@ -876,43 +876,43 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E8" t="n">
         <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>119.85</v>
+        <v>77.70999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>139.34</v>
+        <v>163.89</v>
       </c>
       <c r="H8" t="n">
-        <v>129.59</v>
+        <v>136.72</v>
       </c>
       <c r="I8" t="n">
-        <v>139.34</v>
+        <v>144.18</v>
       </c>
       <c r="J8" t="n">
-        <v>9.75</v>
+        <v>22.68</v>
       </c>
       <c r="K8" t="n">
-        <v>137.39</v>
+        <v>159.92</v>
       </c>
       <c r="L8" t="n">
-        <v>82.8</v>
+        <v>658534.83</v>
       </c>
       <c r="M8" t="n">
-        <v>41.4</v>
+        <v>1554.84</v>
       </c>
       <c r="N8" t="n">
-        <v>41.4</v>
+        <v>25643.27</v>
       </c>
       <c r="O8" t="n">
-        <v>41.4</v>
+        <v>14315.97</v>
       </c>
     </row>
     <row r="9">
@@ -927,10 +927,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E9" t="n">
         <v>100</v>
@@ -978,43 +978,43 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E10" t="n">
-        <v>50</v>
+        <v>95.65000000000001</v>
       </c>
       <c r="F10" t="n">
-        <v>9.42</v>
+        <v>6.68</v>
       </c>
       <c r="G10" t="n">
-        <v>10.1</v>
+        <v>12.03</v>
       </c>
       <c r="H10" t="n">
-        <v>9.76</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>10.1</v>
+        <v>9.5</v>
       </c>
       <c r="J10" t="n">
-        <v>0.34</v>
+        <v>1.59</v>
       </c>
       <c r="K10" t="n">
-        <v>10.03</v>
+        <v>11.81</v>
       </c>
       <c r="L10" t="n">
-        <v>1.49</v>
+        <v>1166.69</v>
       </c>
       <c r="M10" t="n">
-        <v>1.49</v>
+        <v>0.84</v>
       </c>
       <c r="N10" t="n">
-        <v>1.49</v>
+        <v>1081.49</v>
       </c>
       <c r="O10" t="n">
-        <v>1.49</v>
+        <v>55.56</v>
       </c>
     </row>
   </sheetData>
@@ -1028,7 +1028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1070,20 +1070,20 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45662.29166666666</v>
+        <v>45662.29305555556</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45662.33032439081</v>
+        <v>45662.36645138443</v>
       </c>
       <c r="D2" t="n">
-        <v>55.67</v>
+        <v>105.69</v>
       </c>
       <c r="E2" t="n">
-        <v>30.07</v>
+        <v>78.54000000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1094,16 +1094,16 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45662.29305555556</v>
+        <v>45662.29444444444</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45662.35642806848</v>
+        <v>45662.38976335743</v>
       </c>
       <c r="D3" t="n">
-        <v>91.26000000000001</v>
+        <v>137.26</v>
       </c>
       <c r="E3" t="n">
-        <v>66.63</v>
+        <v>110.29</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1118,16 +1118,16 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45662.29583333333</v>
+        <v>45662.29861111111</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45662.35960907352</v>
+        <v>45662.42868614953</v>
       </c>
       <c r="D4" t="n">
-        <v>91.84</v>
+        <v>187.31</v>
       </c>
       <c r="E4" t="n">
-        <v>69.87</v>
+        <v>163.52</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1142,16 +1142,16 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45662.29444444444</v>
+        <v>45662.29722222222</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45662.36259056679</v>
+        <v>45662.44845628603</v>
       </c>
       <c r="D5" t="n">
-        <v>98.13</v>
+        <v>217.78</v>
       </c>
       <c r="E5" t="n">
-        <v>72.23</v>
+        <v>190.43</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1166,16 +1166,16 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45662.29722222222</v>
+        <v>45662.30138888889</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45662.36676671969</v>
+        <v>45662.48071878951</v>
       </c>
       <c r="D6" t="n">
-        <v>100.14</v>
+        <v>258.24</v>
       </c>
       <c r="E6" t="n">
-        <v>72.04000000000001</v>
+        <v>232.47</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1190,16 +1190,16 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45662.29861111111</v>
+        <v>45662.3</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45662.37114121031</v>
+        <v>45662.5065587278</v>
       </c>
       <c r="D7" t="n">
-        <v>104.44</v>
+        <v>297.44</v>
       </c>
       <c r="E7" t="n">
-        <v>76.12</v>
+        <v>266.76</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1214,16 +1214,16 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45662.30138888889</v>
+        <v>45662.30277777778</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45662.37475641909</v>
+        <v>45662.53846813237</v>
       </c>
       <c r="D8" t="n">
-        <v>105.65</v>
+        <v>339.39</v>
       </c>
       <c r="E8" t="n">
-        <v>79.90000000000001</v>
+        <v>312.8</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1241,13 +1241,13 @@
         <v>45662.30416666667</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45662.37855292698</v>
+        <v>45663.31160759155</v>
       </c>
       <c r="D9" t="n">
-        <v>107.12</v>
+        <v>1450.71</v>
       </c>
       <c r="E9" t="n">
-        <v>80.83</v>
+        <v>1424.26</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1262,20 +1262,20 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45662.3</v>
+        <v>45662.30555555555</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45662.50059628971</v>
+        <v>45663.35538182678</v>
       </c>
       <c r="D10" t="n">
-        <v>288.86</v>
+        <v>1511.75</v>
       </c>
       <c r="E10" t="n">
-        <v>35.91</v>
+        <v>1484.22</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1286,20 +1286,2132 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45662.30277777778</v>
+        <v>45662.30972222222</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>45663.30019608489</v>
+        <v>45663.42082936655</v>
       </c>
       <c r="D11" t="n">
-        <v>1436.28</v>
+        <v>1599.99</v>
       </c>
       <c r="E11" t="n">
-        <v>91.56999999999999</v>
+        <v>1572.94</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>45662.31111111111</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>45663.43756760391</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1622.1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1593.55</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>45662.3125</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>45663.45847163483</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1650.2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1626.5</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>45662.29166666666</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>45664.30815304205</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2903.74</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1560.55</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>45662.31388888889</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>45664.32437194397</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2895.1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2866.72</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>45662.31666666667</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>45664.36708358242</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2952.6</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2926.07</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>45662.31805555556</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>45664.3911052832</v>
+      </c>
+      <c r="D17" t="n">
+        <v>2985.19</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2957.56</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>45662.31944444445</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>45664.41210877281</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3013.44</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2990.26</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>45662.29583333333</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>45664.52086205893</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3204.04</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2903.83</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>45662.30694444444</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>45665.38403227897</v>
+      </c>
+      <c r="D20" t="n">
+        <v>4431.01</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4193.1</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>45662.32361111111</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>45665.40692868298</v>
+      </c>
+      <c r="D21" t="n">
+        <v>4439.98</v>
+      </c>
+      <c r="E21" t="n">
+        <v>4409.59</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>45662.325</v>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>45665.43328906162</v>
+      </c>
+      <c r="D22" t="n">
+        <v>4475.94</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4448.8</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>45662.32638888889</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>45665.46620902592</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4521.34</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4493.77</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>45662.32777777778</v>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>45666.29429208017</v>
+      </c>
+      <c r="D24" t="n">
+        <v>5711.78</v>
+      </c>
+      <c r="E24" t="n">
+        <v>5682.46</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>45662.30833333333</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>45666.3040366191</v>
+      </c>
+      <c r="D25" t="n">
+        <v>5753.81</v>
+      </c>
+      <c r="E25" t="n">
+        <v>4449.12</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>45662.32916666667</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>45666.31231671977</v>
+      </c>
+      <c r="D26" t="n">
+        <v>5735.74</v>
+      </c>
+      <c r="E26" t="n">
+        <v>5711.17</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>45662.33055555556</v>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>45666.3440128232</v>
+      </c>
+      <c r="D27" t="n">
+        <v>5779.38</v>
+      </c>
+      <c r="E27" t="n">
+        <v>5751.91</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>45662.33472222222</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>45666.42224247838</v>
+      </c>
+      <c r="D28" t="n">
+        <v>5886.03</v>
+      </c>
+      <c r="E28" t="n">
+        <v>5858.69</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>45662.3375</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>45666.44357719753</v>
+      </c>
+      <c r="D29" t="n">
+        <v>5912.75</v>
+      </c>
+      <c r="E29" t="n">
+        <v>5887.26</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>45662.33611111111</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>45666.48088651554</v>
+      </c>
+      <c r="D30" t="n">
+        <v>5968.48</v>
+      </c>
+      <c r="E30" t="n">
+        <v>5939.26</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>45662.31527777778</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>45667.30684073463</v>
+      </c>
+      <c r="D31" t="n">
+        <v>7187.85</v>
+      </c>
+      <c r="E31" t="n">
+        <v>5865.73</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>45662.32222222222</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>45667.40033280636</v>
+      </c>
+      <c r="D32" t="n">
+        <v>7312.48</v>
+      </c>
+      <c r="E32" t="n">
+        <v>7040.8</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>45662.34027777778</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>45667.41567139886</v>
+      </c>
+      <c r="D33" t="n">
+        <v>7308.57</v>
+      </c>
+      <c r="E33" t="n">
+        <v>7280.98</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>45662.32083333333</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>45667.53905372047</v>
+      </c>
+      <c r="D34" t="n">
+        <v>7514.24</v>
+      </c>
+      <c r="E34" t="n">
+        <v>7189.18</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>45662.34166666667</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>45668.37213282687</v>
+      </c>
+      <c r="D35" t="n">
+        <v>8683.870000000001</v>
+      </c>
+      <c r="E35" t="n">
+        <v>8652.77</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>45662.5125</v>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>45668.37665576444</v>
+      </c>
+      <c r="D36" t="n">
+        <v>8444.379999999999</v>
+      </c>
+      <c r="E36" t="n">
+        <v>7223.66</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>45662.33333333334</v>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>45669.29813801696</v>
+      </c>
+      <c r="D37" t="n">
+        <v>10029.32</v>
+      </c>
+      <c r="E37" t="n">
+        <v>8700.139999999999</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>45662.33194444444</v>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>45669.44341529907</v>
+      </c>
+      <c r="D38" t="n">
+        <v>10240.52</v>
+      </c>
+      <c r="E38" t="n">
+        <v>8867.91</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>45662.33888888889</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>45670.29917730377</v>
+      </c>
+      <c r="D39" t="n">
+        <v>11462.82</v>
+      </c>
+      <c r="E39" t="n">
+        <v>10140.18</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>45662.34305555555</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>45670.30530554261</v>
+      </c>
+      <c r="D40" t="n">
+        <v>11465.64</v>
+      </c>
+      <c r="E40" t="n">
+        <v>9241.959999999999</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>45662.34444444445</v>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>45670.39254016999</v>
+      </c>
+      <c r="D41" t="n">
+        <v>11589.26</v>
+      </c>
+      <c r="E41" t="n">
+        <v>10333.17</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>45662.34583333333</v>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>45670.49629648884</v>
+      </c>
+      <c r="D42" t="n">
+        <v>11736.67</v>
+      </c>
+      <c r="E42" t="n">
+        <v>10466.77</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>45662.67638888889</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>45671.40506611325</v>
+      </c>
+      <c r="D43" t="n">
+        <v>12569.3</v>
+      </c>
+      <c r="E43" t="n">
+        <v>10412.57</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>45662.34722222222</v>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>45671.4442688503</v>
+      </c>
+      <c r="D44" t="n">
+        <v>13099.75</v>
+      </c>
+      <c r="E44" t="n">
+        <v>11994.14</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="n">
+        <v>45662.65416666667</v>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>45672.41320499728</v>
+      </c>
+      <c r="D45" t="n">
+        <v>14053.02</v>
+      </c>
+      <c r="E45" t="n">
+        <v>11856.79</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>45662.83611111111</v>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>45673.39680912522</v>
+      </c>
+      <c r="D46" t="n">
+        <v>15207.41</v>
+      </c>
+      <c r="E46" t="n">
+        <v>13206.89</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>45662.34861111111</v>
+      </c>
+      <c r="C47" s="2" t="n">
+        <v>45678.53756186798</v>
+      </c>
+      <c r="D47" t="n">
+        <v>23312.09</v>
+      </c>
+      <c r="E47" t="n">
+        <v>23285.71</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>45662.35138888889</v>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>45678.54159214268</v>
+      </c>
+      <c r="D48" t="n">
+        <v>23313.89</v>
+      </c>
+      <c r="E48" t="n">
+        <v>23289.18</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>45662.35277777778</v>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>45679.29166666666</v>
+      </c>
+      <c r="D49" t="n">
+        <v>24392</v>
+      </c>
+      <c r="E49" t="n">
+        <v>23286.55</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="n">
+        <v>45662.35555555556</v>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>45679.29528940734</v>
+      </c>
+      <c r="D50" t="n">
+        <v>24393.22</v>
+      </c>
+      <c r="E50" t="n">
+        <v>24363.93</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>45662.35694444444</v>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>45679.29823183955</v>
+      </c>
+      <c r="D51" t="n">
+        <v>24395.45</v>
+      </c>
+      <c r="E51" t="n">
+        <v>24368.49</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="n">
+        <v>45662.35833333333</v>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>45679.30286373736</v>
+      </c>
+      <c r="D52" t="n">
+        <v>24400.12</v>
+      </c>
+      <c r="E52" t="n">
+        <v>24371.5</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
+        <v>45662.35972222222</v>
+      </c>
+      <c r="C53" s="2" t="n">
+        <v>45679.30733133603</v>
+      </c>
+      <c r="D53" t="n">
+        <v>24404.56</v>
+      </c>
+      <c r="E53" t="n">
+        <v>24375.82</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>45662.3625</v>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>45679.31113674448</v>
+      </c>
+      <c r="D54" t="n">
+        <v>24406.04</v>
+      </c>
+      <c r="E54" t="n">
+        <v>24377.02</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="n">
+        <v>45662.36388888889</v>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>45679.3156680484</v>
+      </c>
+      <c r="D55" t="n">
+        <v>24410.56</v>
+      </c>
+      <c r="E55" t="n">
+        <v>24381.76</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="n">
+        <v>45662.36666666667</v>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>45679.39527230465</v>
+      </c>
+      <c r="D56" t="n">
+        <v>24521.19</v>
+      </c>
+      <c r="E56" t="n">
+        <v>24498.06</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="n">
+        <v>45662.36805555555</v>
+      </c>
+      <c r="C57" s="2" t="n">
+        <v>45679.39808909513</v>
+      </c>
+      <c r="D57" t="n">
+        <v>24523.25</v>
+      </c>
+      <c r="E57" t="n">
+        <v>24497.84</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="n">
+        <v>45662.36944444444</v>
+      </c>
+      <c r="C58" s="2" t="n">
+        <v>45679.40209335557</v>
+      </c>
+      <c r="D58" t="n">
+        <v>24527.01</v>
+      </c>
+      <c r="E58" t="n">
+        <v>24499.49</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="n">
+        <v>45662.35416666666</v>
+      </c>
+      <c r="C59" s="2" t="n">
+        <v>45679.40457191706</v>
+      </c>
+      <c r="D59" t="n">
+        <v>24552.58</v>
+      </c>
+      <c r="E59" t="n">
+        <v>24334.01</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="n">
+        <v>45662.37222222222</v>
+      </c>
+      <c r="C60" s="2" t="n">
+        <v>45679.4054014357</v>
+      </c>
+      <c r="D60" t="n">
+        <v>24527.78</v>
+      </c>
+      <c r="E60" t="n">
+        <v>24504.72</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="n">
+        <v>45662.37083333333</v>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>45679.47772115074</v>
+      </c>
+      <c r="D61" t="n">
+        <v>24633.92</v>
+      </c>
+      <c r="E61" t="n">
+        <v>24606.84</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>45662.37361111111</v>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>45679.48015942366</v>
+      </c>
+      <c r="D62" t="n">
+        <v>24633.43</v>
+      </c>
+      <c r="E62" t="n">
+        <v>24609.86</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="n">
+        <v>45662.37638888889</v>
+      </c>
+      <c r="C63" s="2" t="n">
+        <v>45679.4842906786</v>
+      </c>
+      <c r="D63" t="n">
+        <v>24635.38</v>
+      </c>
+      <c r="E63" t="n">
+        <v>24608.39</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>45662.35</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>45679.48824747477</v>
+      </c>
+      <c r="D64" t="n">
+        <v>24679.08</v>
+      </c>
+      <c r="E64" t="n">
+        <v>24407.38</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="n">
+        <v>45662.37777777778</v>
+      </c>
+      <c r="C65" s="2" t="n">
+        <v>45679.48845420307</v>
+      </c>
+      <c r="D65" t="n">
+        <v>24639.37</v>
+      </c>
+      <c r="E65" t="n">
+        <v>24608.73</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>45662.37916666667</v>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>45679.4929093571</v>
+      </c>
+      <c r="D66" t="n">
+        <v>24643.79</v>
+      </c>
+      <c r="E66" t="n">
+        <v>24613.99</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>45662.38333333333</v>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>45679.49740435466</v>
+      </c>
+      <c r="D67" t="n">
+        <v>24644.26</v>
+      </c>
+      <c r="E67" t="n">
+        <v>24616.11</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>45662.38194444445</v>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>45679.50081486114</v>
+      </c>
+      <c r="D68" t="n">
+        <v>24651.17</v>
+      </c>
+      <c r="E68" t="n">
+        <v>24624.37</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="n">
+        <v>45662.36111111111</v>
+      </c>
+      <c r="C69" s="2" t="n">
+        <v>45680.30615307333</v>
+      </c>
+      <c r="D69" t="n">
+        <v>25840.86</v>
+      </c>
+      <c r="E69" t="n">
+        <v>24520</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>45662.38472222222</v>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>45680.40084635137</v>
+      </c>
+      <c r="D70" t="n">
+        <v>25943.22</v>
+      </c>
+      <c r="E70" t="n">
+        <v>25912.95</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>45662.38611111111</v>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>45680.40517113198</v>
+      </c>
+      <c r="D71" t="n">
+        <v>25947.45</v>
+      </c>
+      <c r="E71" t="n">
+        <v>25921.01</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>45662.36527777778</v>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v>45680.40836026006</v>
+      </c>
+      <c r="D72" t="n">
+        <v>25982.04</v>
+      </c>
+      <c r="E72" t="n">
+        <v>25666.25</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="n">
+        <v>45662.3875</v>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>45680.40967682941</v>
+      </c>
+      <c r="D73" t="n">
+        <v>25951.93</v>
+      </c>
+      <c r="E73" t="n">
+        <v>25924.95</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>45662.38055555556</v>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v>45680.5357645696</v>
+      </c>
+      <c r="D74" t="n">
+        <v>26143.5</v>
+      </c>
+      <c r="E74" t="n">
+        <v>25832.45</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="n">
+        <v>45662.375</v>
+      </c>
+      <c r="C75" s="2" t="n">
+        <v>45681.29936357489</v>
+      </c>
+      <c r="D75" t="n">
+        <v>27251.08</v>
+      </c>
+      <c r="E75" t="n">
+        <v>25950.42</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>45662.38888888889</v>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>45681.3021171319</v>
+      </c>
+      <c r="D76" t="n">
+        <v>27235.05</v>
+      </c>
+      <c r="E76" t="n">
+        <v>27208.32</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="n">
+        <v>45662.39027777778</v>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>45681.30630891504</v>
+      </c>
+      <c r="D77" t="n">
+        <v>27239.08</v>
+      </c>
+      <c r="E77" t="n">
+        <v>27211.24</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>45662.39166666667</v>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>45681.30929125974</v>
+      </c>
+      <c r="D78" t="n">
+        <v>27241.38</v>
+      </c>
+      <c r="E78" t="n">
+        <v>27213.53</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="n">
+        <v>45662.39305555556</v>
+      </c>
+      <c r="C79" s="2" t="n">
+        <v>45681.31366135218</v>
+      </c>
+      <c r="D79" t="n">
+        <v>27245.67</v>
+      </c>
+      <c r="E79" t="n">
+        <v>27217.19</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>45662.39444444444</v>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v>45681.31803175672</v>
+      </c>
+      <c r="D80" t="n">
+        <v>27249.97</v>
+      </c>
+      <c r="E80" t="n">
+        <v>27222.06</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="n">
+        <v>45662.39722222222</v>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>45681.3209855744</v>
+      </c>
+      <c r="D81" t="n">
+        <v>27250.22</v>
+      </c>
+      <c r="E81" t="n">
+        <v>27225.54</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>45662.39861111111</v>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>45681.3242839368</v>
+      </c>
+      <c r="D82" t="n">
+        <v>27252.97</v>
+      </c>
+      <c r="E82" t="n">
+        <v>27226.11</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="n">
+        <v>45662.4</v>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v>45681.32760307437</v>
+      </c>
+      <c r="D83" t="n">
+        <v>27255.75</v>
+      </c>
+      <c r="E83" t="n">
+        <v>27231.83</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>45662.40277777778</v>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>45681.33119633021</v>
+      </c>
+      <c r="D84" t="n">
+        <v>27256.92</v>
+      </c>
+      <c r="E84" t="n">
+        <v>27228.59</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="n">
+        <v>45662.40555555555</v>
+      </c>
+      <c r="C85" s="2" t="n">
+        <v>45681.33461168112</v>
+      </c>
+      <c r="D85" t="n">
+        <v>27257.84</v>
+      </c>
+      <c r="E85" t="n">
+        <v>27235.5</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="n">
+        <v>45662.40416666667</v>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>45681.33846355641</v>
+      </c>
+      <c r="D86" t="n">
+        <v>27265.39</v>
+      </c>
+      <c r="E86" t="n">
+        <v>27234.89</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="n">
+        <v>45662.40694444445</v>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v>45681.34197540774</v>
+      </c>
+      <c r="D87" t="n">
+        <v>27266.44</v>
+      </c>
+      <c r="E87" t="n">
+        <v>27237.76</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="n">
+        <v>45662.40833333333</v>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>45681.34628781332</v>
+      </c>
+      <c r="D88" t="n">
+        <v>27270.65</v>
+      </c>
+      <c r="E88" t="n">
+        <v>27242.27</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="n">
+        <v>45662.40972222222</v>
+      </c>
+      <c r="C89" s="2" t="n">
+        <v>45681.34972006597</v>
+      </c>
+      <c r="D89" t="n">
+        <v>27273.6</v>
+      </c>
+      <c r="E89" t="n">
+        <v>27244.35</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n">
+        <v>45662.4125</v>
+      </c>
+      <c r="C90" s="2" t="n">
+        <v>45681.35353542436</v>
+      </c>
+      <c r="D90" t="n">
+        <v>27275.09</v>
+      </c>
+      <c r="E90" t="n">
+        <v>27248.95</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="n">
+        <v>45662.41388888889</v>
+      </c>
+      <c r="C91" s="2" t="n">
+        <v>45681.35595963308</v>
+      </c>
+      <c r="D91" t="n">
+        <v>27276.58</v>
+      </c>
+      <c r="E91" t="n">
+        <v>27248.41</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="n">
+        <v>45662.41527777778</v>
+      </c>
+      <c r="C92" s="2" t="n">
+        <v>45681.36052819547</v>
+      </c>
+      <c r="D92" t="n">
+        <v>27281.16</v>
+      </c>
+      <c r="E92" t="n">
+        <v>27254.37</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="n">
+        <v>45662.41111111111</v>
+      </c>
+      <c r="C93" s="2" t="n">
+        <v>45682.4118632898</v>
+      </c>
+      <c r="D93" t="n">
+        <v>28801.08</v>
+      </c>
+      <c r="E93" t="n">
+        <v>28502.08</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="n">
+        <v>45662.41666666666</v>
+      </c>
+      <c r="C94" s="2" t="n">
+        <v>45682.41508173538</v>
+      </c>
+      <c r="D94" t="n">
+        <v>28797.72</v>
+      </c>
+      <c r="E94" t="n">
+        <v>28772.41</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="n">
+        <v>45662.41805555556</v>
+      </c>
+      <c r="C95" s="2" t="n">
+        <v>45682.41875947017</v>
+      </c>
+      <c r="D95" t="n">
+        <v>28801.01</v>
+      </c>
+      <c r="E95" t="n">
+        <v>28775.32</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="n">
+        <v>45662.41944444444</v>
+      </c>
+      <c r="C96" s="2" t="n">
+        <v>45682.42328160448</v>
+      </c>
+      <c r="D96" t="n">
+        <v>28805.53</v>
+      </c>
+      <c r="E96" t="n">
+        <v>28777.75</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="n">
+        <v>45662.42361111111</v>
+      </c>
+      <c r="C97" s="2" t="n">
+        <v>45682.42780392143</v>
+      </c>
+      <c r="D97" t="n">
+        <v>28806.04</v>
+      </c>
+      <c r="E97" t="n">
+        <v>28781.2</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="n">
+        <v>45662.42222222222</v>
+      </c>
+      <c r="C98" s="2" t="n">
+        <v>45682.50846915448</v>
+      </c>
+      <c r="D98" t="n">
+        <v>28924.2</v>
+      </c>
+      <c r="E98" t="n">
+        <v>27819.88</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="n">
+        <v>45662.425</v>
+      </c>
+      <c r="C99" s="2" t="n">
+        <v>45682.511289335</v>
+      </c>
+      <c r="D99" t="n">
+        <v>28924.26</v>
+      </c>
+      <c r="E99" t="n">
+        <v>28903.7</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1336,7 +3448,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>500</v>
       </c>
     </row>
     <row r="3">
@@ -1346,7 +3458,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4">
@@ -1356,7 +3468,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50</v>
+        <v>95.65000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -1366,7 +3478,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9.76</v>
+        <v>9.710000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -1376,7 +3488,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10.03</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="7">
@@ -1386,7 +3498,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.49</v>
+        <v>55.56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Still need to fix simulation to properly take into account the value for simulation days.
</commit_message>
<xml_diff>
--- a/5.5.13 Real Property-Monthly Reviews-2_results.xlsx
+++ b/5.5.13 Real Property-Monthly Reviews-2_results.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>29.79</v>
+        <v>4.36</v>
       </c>
     </row>
     <row r="3">
@@ -464,7 +464,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.5</v>
+        <v>0.09</v>
       </c>
     </row>
   </sheetData>
@@ -573,40 +573,40 @@
         <v>500</v>
       </c>
       <c r="D2" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="E2" t="n">
-        <v>19.6</v>
+        <v>24.8</v>
       </c>
       <c r="F2" t="n">
-        <v>105.69</v>
+        <v>59.95</v>
       </c>
       <c r="G2" t="n">
-        <v>28924.26</v>
+        <v>31612.33</v>
       </c>
       <c r="H2" t="n">
-        <v>16728.64</v>
+        <v>18879.43</v>
       </c>
       <c r="I2" t="n">
-        <v>24395.45</v>
+        <v>23077.82</v>
       </c>
       <c r="J2" t="n">
-        <v>10682.1</v>
+        <v>10449.24</v>
       </c>
       <c r="K2" t="n">
-        <v>27274.05</v>
+        <v>30030.93</v>
       </c>
       <c r="L2" t="n">
-        <v>1608681.15</v>
+        <v>2304145.7</v>
       </c>
       <c r="M2" t="n">
-        <v>78.54000000000001</v>
+        <v>32.97</v>
       </c>
       <c r="N2" t="n">
-        <v>28903.7</v>
+        <v>31276.63</v>
       </c>
       <c r="O2" t="n">
-        <v>16415.11</v>
+        <v>18581.82</v>
       </c>
     </row>
     <row r="3">
@@ -672,43 +672,43 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="D4" t="n">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>5.12</v>
+        <v>5.19</v>
       </c>
       <c r="G4" t="n">
         <v>9.58</v>
       </c>
       <c r="H4" t="n">
-        <v>8.029999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="I4" t="n">
-        <v>8.18</v>
+        <v>8.24</v>
       </c>
       <c r="J4" t="n">
-        <v>1.1</v>
+        <v>1.04</v>
       </c>
       <c r="K4" t="n">
-        <v>9.34</v>
+        <v>9.35</v>
       </c>
       <c r="L4" t="n">
-        <v>12164872.29</v>
+        <v>10183752.51</v>
       </c>
       <c r="M4" t="n">
-        <v>5.71</v>
+        <v>6.21</v>
       </c>
       <c r="N4" t="n">
-        <v>21931.43</v>
+        <v>20332.4</v>
       </c>
       <c r="O4" t="n">
-        <v>12238.3</v>
+        <v>10255.54</v>
       </c>
     </row>
     <row r="5">
@@ -723,10 +723,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="D5" t="n">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="E5" t="n">
         <v>100</v>
@@ -774,43 +774,43 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="D6" t="n">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>3.4</v>
+        <v>3.42</v>
       </c>
       <c r="G6" t="n">
-        <v>6.71</v>
+        <v>6.73</v>
       </c>
       <c r="H6" t="n">
-        <v>5.46</v>
+        <v>5.53</v>
       </c>
       <c r="I6" t="n">
-        <v>5.49</v>
+        <v>5.65</v>
       </c>
       <c r="J6" t="n">
-        <v>0.92</v>
+        <v>0.82</v>
       </c>
       <c r="K6" t="n">
-        <v>6.58</v>
+        <v>6.55</v>
       </c>
       <c r="L6" t="n">
-        <v>2459394.43</v>
+        <v>3098701.11</v>
       </c>
       <c r="M6" t="n">
-        <v>72.83</v>
+        <v>32.97</v>
       </c>
       <c r="N6" t="n">
-        <v>25765.28</v>
+        <v>27225.48</v>
       </c>
       <c r="O6" t="n">
-        <v>16287.38</v>
+        <v>16570.59</v>
       </c>
     </row>
     <row r="7">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="D7" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
       <c r="E7" t="n">
         <v>100</v>
@@ -852,16 +852,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>9.32</v>
+        <v>8.57</v>
       </c>
       <c r="M7" t="n">
-        <v>9.32</v>
+        <v>8.57</v>
       </c>
       <c r="N7" t="n">
-        <v>9.32</v>
+        <v>8.57</v>
       </c>
       <c r="O7" t="n">
-        <v>9.32</v>
+        <v>8.57</v>
       </c>
     </row>
     <row r="8">
@@ -876,43 +876,43 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D8" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E8" t="n">
         <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>77.70999999999999</v>
+        <v>70.27</v>
       </c>
       <c r="G8" t="n">
-        <v>163.89</v>
+        <v>161.49</v>
       </c>
       <c r="H8" t="n">
-        <v>136.72</v>
+        <v>126.06</v>
       </c>
       <c r="I8" t="n">
-        <v>144.18</v>
+        <v>133.75</v>
       </c>
       <c r="J8" t="n">
-        <v>22.68</v>
+        <v>27.1</v>
       </c>
       <c r="K8" t="n">
-        <v>159.92</v>
+        <v>156.43</v>
       </c>
       <c r="L8" t="n">
-        <v>658534.83</v>
+        <v>1031770.38</v>
       </c>
       <c r="M8" t="n">
-        <v>1554.84</v>
+        <v>1510.3</v>
       </c>
       <c r="N8" t="n">
-        <v>25643.27</v>
+        <v>27125.38</v>
       </c>
       <c r="O8" t="n">
-        <v>14315.97</v>
+        <v>19106.86</v>
       </c>
     </row>
     <row r="9">
@@ -927,10 +927,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D9" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E9" t="n">
         <v>100</v>
@@ -978,43 +978,43 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D10" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="E10" t="n">
-        <v>95.65000000000001</v>
+        <v>96.77</v>
       </c>
       <c r="F10" t="n">
-        <v>6.68</v>
+        <v>7.59</v>
       </c>
       <c r="G10" t="n">
-        <v>12.03</v>
+        <v>12.07</v>
       </c>
       <c r="H10" t="n">
-        <v>9.710000000000001</v>
+        <v>10.36</v>
       </c>
       <c r="I10" t="n">
-        <v>9.5</v>
+        <v>10.58</v>
       </c>
       <c r="J10" t="n">
-        <v>1.59</v>
+        <v>1.27</v>
       </c>
       <c r="K10" t="n">
-        <v>11.81</v>
+        <v>11.85</v>
       </c>
       <c r="L10" t="n">
-        <v>1166.69</v>
+        <v>129.44</v>
       </c>
       <c r="M10" t="n">
-        <v>0.84</v>
+        <v>0.75</v>
       </c>
       <c r="N10" t="n">
-        <v>1081.49</v>
+        <v>6.83</v>
       </c>
       <c r="O10" t="n">
-        <v>55.56</v>
+        <v>4.46</v>
       </c>
     </row>
   </sheetData>
@@ -1028,7 +1028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1070,20 +1070,20 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45662.29305555556</v>
+        <v>45662.29166666666</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45662.36645138443</v>
+        <v>45662.33329752198</v>
       </c>
       <c r="D2" t="n">
-        <v>105.69</v>
+        <v>59.95</v>
       </c>
       <c r="E2" t="n">
-        <v>78.54000000000001</v>
+        <v>32.97</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1094,16 +1094,16 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45662.29444444444</v>
+        <v>45662.29305555556</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45662.38976335743</v>
+        <v>45662.37334402597</v>
       </c>
       <c r="D3" t="n">
-        <v>137.26</v>
+        <v>115.62</v>
       </c>
       <c r="E3" t="n">
-        <v>110.29</v>
+        <v>87.23</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1118,16 +1118,16 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45662.29861111111</v>
+        <v>45662.29583333333</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45662.42868614953</v>
+        <v>45662.40163947275</v>
       </c>
       <c r="D4" t="n">
-        <v>187.31</v>
+        <v>152.36</v>
       </c>
       <c r="E4" t="n">
-        <v>163.52</v>
+        <v>125.87</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -1145,13 +1145,13 @@
         <v>45662.29722222222</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45662.44845628603</v>
+        <v>45662.43762263396</v>
       </c>
       <c r="D5" t="n">
-        <v>217.78</v>
+        <v>202.18</v>
       </c>
       <c r="E5" t="n">
-        <v>190.43</v>
+        <v>179.17</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1166,16 +1166,16 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45662.30138888889</v>
+        <v>45662.29861111111</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45662.48071878951</v>
+        <v>45662.46990041722</v>
       </c>
       <c r="D6" t="n">
-        <v>258.24</v>
+        <v>246.66</v>
       </c>
       <c r="E6" t="n">
-        <v>232.47</v>
+        <v>219.67</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1193,13 +1193,13 @@
         <v>45662.3</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45662.5065587278</v>
+        <v>45662.51885033459</v>
       </c>
       <c r="D7" t="n">
-        <v>297.44</v>
+        <v>315.14</v>
       </c>
       <c r="E7" t="n">
-        <v>266.76</v>
+        <v>285.13</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1214,16 +1214,16 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45662.30277777778</v>
+        <v>45662.30138888889</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45662.53846813237</v>
+        <v>45662.5399183164</v>
       </c>
       <c r="D8" t="n">
-        <v>339.39</v>
+        <v>343.48</v>
       </c>
       <c r="E8" t="n">
-        <v>312.8</v>
+        <v>316.25</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1238,16 +1238,16 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45662.30416666667</v>
+        <v>45662.30277777778</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45663.31160759155</v>
+        <v>45663.31580679751</v>
       </c>
       <c r="D9" t="n">
-        <v>1450.71</v>
+        <v>1458.76</v>
       </c>
       <c r="E9" t="n">
-        <v>1424.26</v>
+        <v>1431.38</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1262,16 +1262,16 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45662.30555555555</v>
+        <v>45662.30416666667</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45663.35538182678</v>
+        <v>45663.35101653879</v>
       </c>
       <c r="D10" t="n">
-        <v>1511.75</v>
+        <v>1507.46</v>
       </c>
       <c r="E10" t="n">
-        <v>1484.22</v>
+        <v>1480.52</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1286,16 +1286,16 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45662.30972222222</v>
+        <v>45662.30555555555</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>45663.42082936655</v>
+        <v>45663.39079347986</v>
       </c>
       <c r="D11" t="n">
-        <v>1599.99</v>
+        <v>1562.74</v>
       </c>
       <c r="E11" t="n">
-        <v>1572.94</v>
+        <v>1532.57</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1310,16 +1310,16 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45662.31111111111</v>
+        <v>45662.30833333333</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>45663.43756760391</v>
+        <v>45663.43154756449</v>
       </c>
       <c r="D12" t="n">
-        <v>1622.1</v>
+        <v>1617.43</v>
       </c>
       <c r="E12" t="n">
-        <v>1593.55</v>
+        <v>1589.82</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1334,20 +1334,20 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45662.3125</v>
+        <v>45662.29444444444</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>45663.45847163483</v>
+        <v>45663.5338707749</v>
       </c>
       <c r="D13" t="n">
-        <v>1650.2</v>
+        <v>1784.77</v>
       </c>
       <c r="E13" t="n">
-        <v>1626.5</v>
+        <v>1532.25</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1358,20 +1358,20 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45662.29166666666</v>
+        <v>45662.31111111111</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>45664.30815304205</v>
+        <v>45664.3203193547</v>
       </c>
       <c r="D14" t="n">
-        <v>2903.74</v>
+        <v>2893.26</v>
       </c>
       <c r="E14" t="n">
-        <v>1560.55</v>
+        <v>2864.74</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1382,16 +1382,16 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>45662.31388888889</v>
+        <v>45662.3125</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>45664.32437194397</v>
+        <v>45664.34962421956</v>
       </c>
       <c r="D15" t="n">
-        <v>2895.1</v>
+        <v>2933.46</v>
       </c>
       <c r="E15" t="n">
-        <v>2866.72</v>
+        <v>2907.38</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1406,16 +1406,16 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45662.31666666667</v>
+        <v>45662.31527777778</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45664.36708358242</v>
+        <v>45664.41355094349</v>
       </c>
       <c r="D16" t="n">
-        <v>2952.6</v>
+        <v>3021.51</v>
       </c>
       <c r="E16" t="n">
-        <v>2926.07</v>
+        <v>2990.55</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1430,16 +1430,16 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>45662.31805555556</v>
+        <v>45662.31666666667</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>45664.3911052832</v>
+        <v>45664.43969734229</v>
       </c>
       <c r="D17" t="n">
-        <v>2985.19</v>
+        <v>3057.16</v>
       </c>
       <c r="E17" t="n">
-        <v>2957.56</v>
+        <v>3029.78</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1454,16 +1454,16 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45662.31944444445</v>
+        <v>45662.31805555556</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>45664.41210877281</v>
+        <v>45664.46696351265</v>
       </c>
       <c r="D18" t="n">
-        <v>3013.44</v>
+        <v>3094.43</v>
       </c>
       <c r="E18" t="n">
-        <v>2990.26</v>
+        <v>3065.71</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1478,20 +1478,20 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>45662.29583333333</v>
+        <v>45662.32222222222</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>45664.52086205893</v>
+        <v>45665.30706725767</v>
       </c>
       <c r="D19" t="n">
-        <v>3204.04</v>
+        <v>4298.18</v>
       </c>
       <c r="E19" t="n">
-        <v>2903.83</v>
+        <v>4270.89</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1502,20 +1502,20 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>45662.30694444444</v>
+        <v>45662.32361111111</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>45665.38403227897</v>
+        <v>45665.33880627694</v>
       </c>
       <c r="D20" t="n">
-        <v>4431.01</v>
+        <v>4341.88</v>
       </c>
       <c r="E20" t="n">
-        <v>4193.1</v>
+        <v>4312.75</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1526,16 +1526,16 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>45662.32361111111</v>
+        <v>45662.325</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>45665.40692868298</v>
+        <v>45665.36845109234</v>
       </c>
       <c r="D21" t="n">
-        <v>4439.98</v>
+        <v>4382.57</v>
       </c>
       <c r="E21" t="n">
-        <v>4409.59</v>
+        <v>4353.12</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1550,20 +1550,20 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>45662.325</v>
+        <v>45662.31388888889</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>45665.43328906162</v>
+        <v>45665.49950817604</v>
       </c>
       <c r="D22" t="n">
-        <v>4475.94</v>
+        <v>4587.29</v>
       </c>
       <c r="E22" t="n">
-        <v>4448.8</v>
+        <v>4318.61</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1574,20 +1574,20 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>45662.32638888889</v>
+        <v>45662.30694444444</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>45665.46620902592</v>
+        <v>45666.30669177544</v>
       </c>
       <c r="D23" t="n">
-        <v>4521.34</v>
+        <v>5759.64</v>
       </c>
       <c r="E23" t="n">
-        <v>4493.77</v>
+        <v>4419.3</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1601,13 +1601,13 @@
         <v>45662.32777777778</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>45666.29429208017</v>
+        <v>45666.31027586611</v>
       </c>
       <c r="D24" t="n">
-        <v>5711.78</v>
+        <v>5734.8</v>
       </c>
       <c r="E24" t="n">
-        <v>5682.46</v>
+        <v>5711.16</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1622,20 +1622,20 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>45662.30833333333</v>
+        <v>45662.32638888889</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>45666.3040366191</v>
+        <v>45666.33877452159</v>
       </c>
       <c r="D25" t="n">
-        <v>5753.81</v>
+        <v>5777.84</v>
       </c>
       <c r="E25" t="n">
-        <v>4449.12</v>
+        <v>5749.81</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1649,13 +1649,13 @@
         <v>45662.32916666667</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>45666.31231671977</v>
+        <v>45666.3760189571</v>
       </c>
       <c r="D26" t="n">
-        <v>5735.74</v>
+        <v>5827.47</v>
       </c>
       <c r="E26" t="n">
-        <v>5711.17</v>
+        <v>5797.79</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1670,16 +1670,16 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45662.33055555556</v>
+        <v>45662.33194444444</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>45666.3440128232</v>
+        <v>45666.39543306366</v>
       </c>
       <c r="D27" t="n">
-        <v>5779.38</v>
+        <v>5851.42</v>
       </c>
       <c r="E27" t="n">
-        <v>5751.91</v>
+        <v>5825.24</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1694,16 +1694,16 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45662.33472222222</v>
+        <v>45662.33055555556</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>45666.42224247838</v>
+        <v>45666.4291758629</v>
       </c>
       <c r="D28" t="n">
-        <v>5886.03</v>
+        <v>5902.01</v>
       </c>
       <c r="E28" t="n">
-        <v>5858.69</v>
+        <v>5873.09</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1718,16 +1718,16 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45662.3375</v>
+        <v>45662.33333333334</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>45666.44357719753</v>
+        <v>45666.44954801867</v>
       </c>
       <c r="D29" t="n">
-        <v>5912.75</v>
+        <v>5927.35</v>
       </c>
       <c r="E29" t="n">
-        <v>5887.26</v>
+        <v>5901.38</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1742,20 +1742,20 @@
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45662.33611111111</v>
+        <v>45662.30972222222</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>45666.48088651554</v>
+        <v>45667.30633220963</v>
       </c>
       <c r="D30" t="n">
-        <v>5968.48</v>
+        <v>7195.12</v>
       </c>
       <c r="E30" t="n">
-        <v>5939.26</v>
+        <v>5796.98</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1766,16 +1766,16 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45662.31527777778</v>
+        <v>45662.48888888889</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>45667.30684073463</v>
+        <v>45667.37023438902</v>
       </c>
       <c r="D31" t="n">
-        <v>7187.85</v>
+        <v>7029.14</v>
       </c>
       <c r="E31" t="n">
-        <v>5865.73</v>
+        <v>5687.5</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1790,16 +1790,16 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45662.32222222222</v>
+        <v>45662.32083333333</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>45667.40033280636</v>
+        <v>45667.47586051536</v>
       </c>
       <c r="D32" t="n">
-        <v>7312.48</v>
+        <v>7423.24</v>
       </c>
       <c r="E32" t="n">
-        <v>7040.8</v>
+        <v>7158.56</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1814,16 +1814,16 @@
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45662.34027777778</v>
+        <v>45662.33611111111</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>45667.41567139886</v>
+        <v>45667.48772982143</v>
       </c>
       <c r="D33" t="n">
-        <v>7308.57</v>
+        <v>7418.33</v>
       </c>
       <c r="E33" t="n">
-        <v>7280.98</v>
+        <v>7389.91</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1838,20 +1838,20 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45662.32083333333</v>
+        <v>45662.3375</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>45667.53905372047</v>
+        <v>45667.52647083604</v>
       </c>
       <c r="D34" t="n">
-        <v>7514.24</v>
+        <v>7472.12</v>
       </c>
       <c r="E34" t="n">
-        <v>7189.18</v>
+        <v>7444.75</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1862,16 +1862,16 @@
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45662.34166666667</v>
+        <v>45662.34027777778</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>45668.37213282687</v>
+        <v>45668.41375448016</v>
       </c>
       <c r="D35" t="n">
-        <v>8683.870000000001</v>
+        <v>8745.809999999999</v>
       </c>
       <c r="E35" t="n">
-        <v>8652.77</v>
+        <v>8720.639999999999</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1886,16 +1886,16 @@
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45662.5125</v>
+        <v>45662.31944444445</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>45668.37665576444</v>
+        <v>45668.41976485375</v>
       </c>
       <c r="D36" t="n">
-        <v>8444.379999999999</v>
+        <v>8784.459999999999</v>
       </c>
       <c r="E36" t="n">
-        <v>7223.66</v>
+        <v>8457.84</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1910,20 +1910,20 @@
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45662.33333333334</v>
+        <v>45662.33888888889</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>45669.29813801696</v>
+        <v>45668.44414685827</v>
       </c>
       <c r="D37" t="n">
-        <v>10029.32</v>
+        <v>8791.57</v>
       </c>
       <c r="E37" t="n">
-        <v>8700.139999999999</v>
+        <v>8764.33</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1934,20 +1934,20 @@
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45662.33194444444</v>
+        <v>45662.34166666667</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>45669.44341529907</v>
+        <v>45668.4639501508</v>
       </c>
       <c r="D38" t="n">
-        <v>10240.52</v>
+        <v>8816.09</v>
       </c>
       <c r="E38" t="n">
-        <v>8867.91</v>
+        <v>8794.24</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1958,20 +1958,20 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45662.33888888889</v>
+        <v>45662.34305555555</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>45670.29917730377</v>
+        <v>45668.50091386359</v>
       </c>
       <c r="D39" t="n">
-        <v>11462.82</v>
+        <v>8867.32</v>
       </c>
       <c r="E39" t="n">
-        <v>10140.18</v>
+        <v>8841.049999999999</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -1982,16 +1982,16 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45662.34305555555</v>
+        <v>45662.33472222222</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>45670.30530554261</v>
+        <v>45669.30678219995</v>
       </c>
       <c r="D40" t="n">
-        <v>11465.64</v>
+        <v>10039.77</v>
       </c>
       <c r="E40" t="n">
-        <v>9241.959999999999</v>
+        <v>7766.26</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -2009,17 +2009,17 @@
         <v>45662.34444444445</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>45670.39254016999</v>
+        <v>45669.53506792918</v>
       </c>
       <c r="D41" t="n">
-        <v>11589.26</v>
+        <v>10354.5</v>
       </c>
       <c r="E41" t="n">
-        <v>10333.17</v>
+        <v>9250.26</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2030,20 +2030,20 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45662.34583333333</v>
+        <v>45662.85138888889</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>45670.49629648884</v>
+        <v>45670.41012530989</v>
       </c>
       <c r="D42" t="n">
-        <v>11736.67</v>
+        <v>10884.58</v>
       </c>
       <c r="E42" t="n">
-        <v>10466.77</v>
+        <v>8970.440000000001</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2054,16 +2054,16 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45662.67638888889</v>
+        <v>45662.69305555556</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>45671.40506611325</v>
+        <v>45674.41309944067</v>
       </c>
       <c r="D43" t="n">
-        <v>12569.3</v>
+        <v>16876.86</v>
       </c>
       <c r="E43" t="n">
-        <v>10412.57</v>
+        <v>14727.07</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -2078,20 +2078,20 @@
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45662.34722222222</v>
+        <v>45662.88472222222</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>45671.4442688503</v>
+        <v>45675.41094876696</v>
       </c>
       <c r="D44" t="n">
-        <v>13099.75</v>
+        <v>18037.77</v>
       </c>
       <c r="E44" t="n">
-        <v>11994.14</v>
+        <v>16140.3</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2102,20 +2102,20 @@
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45662.65416666667</v>
+        <v>45662.83333333334</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>45672.41320499728</v>
+        <v>45677.36096354036</v>
       </c>
       <c r="D45" t="n">
-        <v>14053.02</v>
+        <v>20919.79</v>
       </c>
       <c r="E45" t="n">
-        <v>11856.79</v>
+        <v>19061.21</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2126,20 +2126,20 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45662.83611111111</v>
+        <v>45662.34722222222</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>45673.39680912522</v>
+        <v>45677.42750575664</v>
       </c>
       <c r="D46" t="n">
-        <v>15207.41</v>
+        <v>21715.61</v>
       </c>
       <c r="E46" t="n">
-        <v>13206.89</v>
+        <v>21688.09</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2153,13 +2153,13 @@
         <v>45662.34861111111</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>45678.53756186798</v>
+        <v>45677.43048310962</v>
       </c>
       <c r="D47" t="n">
-        <v>23312.09</v>
+        <v>21717.9</v>
       </c>
       <c r="E47" t="n">
-        <v>23285.71</v>
+        <v>21691.41</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2174,16 +2174,16 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45662.35138888889</v>
+        <v>45662.35</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>45678.54159214268</v>
+        <v>45677.43410099015</v>
       </c>
       <c r="D48" t="n">
-        <v>23313.89</v>
+        <v>21721.11</v>
       </c>
       <c r="E48" t="n">
-        <v>23289.18</v>
+        <v>21695.68</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2198,16 +2198,16 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45662.35277777778</v>
+        <v>45662.35138888889</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>45679.29166666666</v>
+        <v>45677.43877493078</v>
       </c>
       <c r="D49" t="n">
-        <v>24392</v>
+        <v>21725.84</v>
       </c>
       <c r="E49" t="n">
-        <v>23286.55</v>
+        <v>21696.42</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2222,16 +2222,16 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>45662.35555555556</v>
+        <v>45662.35277777778</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>45679.29528940734</v>
+        <v>45677.44257253456</v>
       </c>
       <c r="D50" t="n">
-        <v>24393.22</v>
+        <v>21729.3</v>
       </c>
       <c r="E50" t="n">
-        <v>24363.93</v>
+        <v>21703.32</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -2246,16 +2246,16 @@
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>45662.35694444444</v>
+        <v>45662.35555555556</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>45679.29823183955</v>
+        <v>45677.44671235355</v>
       </c>
       <c r="D51" t="n">
-        <v>24395.45</v>
+        <v>21731.27</v>
       </c>
       <c r="E51" t="n">
-        <v>24368.49</v>
+        <v>21705.91</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -2270,16 +2270,16 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>45662.35833333333</v>
+        <v>45662.35694444444</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>45679.30286373736</v>
+        <v>45677.44981649565</v>
       </c>
       <c r="D52" t="n">
-        <v>24400.12</v>
+        <v>21733.74</v>
       </c>
       <c r="E52" t="n">
-        <v>24371.5</v>
+        <v>21706.66</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2297,13 +2297,13 @@
         <v>45662.35972222222</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>45679.30733133603</v>
+        <v>45677.45390445285</v>
       </c>
       <c r="D53" t="n">
-        <v>24404.56</v>
+        <v>21735.62</v>
       </c>
       <c r="E53" t="n">
-        <v>24375.82</v>
+        <v>21707.87</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -2318,16 +2318,16 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>45662.3625</v>
+        <v>45662.36111111111</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>45679.31113674448</v>
+        <v>45677.45685047198</v>
       </c>
       <c r="D54" t="n">
-        <v>24406.04</v>
+        <v>21737.86</v>
       </c>
       <c r="E54" t="n">
-        <v>24377.02</v>
+        <v>21711.54</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2342,16 +2342,16 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>45662.36388888889</v>
+        <v>45662.3625</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>45679.3156680484</v>
+        <v>45677.4611666516</v>
       </c>
       <c r="D55" t="n">
-        <v>24410.56</v>
+        <v>21742.08</v>
       </c>
       <c r="E55" t="n">
-        <v>24381.76</v>
+        <v>21717.84</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2366,16 +2366,16 @@
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>45662.36666666667</v>
+        <v>45662.36388888889</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>45679.39527230465</v>
+        <v>45677.4657679312</v>
       </c>
       <c r="D56" t="n">
-        <v>24521.19</v>
+        <v>21746.71</v>
       </c>
       <c r="E56" t="n">
-        <v>24498.06</v>
+        <v>21719.51</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2390,16 +2390,16 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>45662.36805555555</v>
+        <v>45662.36527777778</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>45679.39808909513</v>
+        <v>45677.46909221537</v>
       </c>
       <c r="D57" t="n">
-        <v>24523.25</v>
+        <v>21749.49</v>
       </c>
       <c r="E57" t="n">
-        <v>24497.84</v>
+        <v>21721.29</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -2414,16 +2414,16 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>45662.36944444444</v>
+        <v>45662.36666666667</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>45679.40209335557</v>
+        <v>45678.29604698024</v>
       </c>
       <c r="D58" t="n">
-        <v>24527.01</v>
+        <v>22938.31</v>
       </c>
       <c r="E58" t="n">
-        <v>24499.49</v>
+        <v>22909.59</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2438,20 +2438,20 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>45662.35416666666</v>
+        <v>45662.36944444444</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>45679.40457191706</v>
+        <v>45678.30023809815</v>
       </c>
       <c r="D59" t="n">
-        <v>24552.58</v>
+        <v>22940.34</v>
       </c>
       <c r="E59" t="n">
-        <v>24334.01</v>
+        <v>22910.68</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2465,13 +2465,13 @@
         <v>45662.37222222222</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>45679.4054014357</v>
+        <v>45678.30489852621</v>
       </c>
       <c r="D60" t="n">
-        <v>24527.78</v>
+        <v>22943.05</v>
       </c>
       <c r="E60" t="n">
-        <v>24504.72</v>
+        <v>22915.49</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -2486,20 +2486,20 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>45662.37083333333</v>
+        <v>45662.34583333333</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>45679.47772115074</v>
+        <v>45678.30506665447</v>
       </c>
       <c r="D61" t="n">
-        <v>24633.92</v>
+        <v>22981.3</v>
       </c>
       <c r="E61" t="n">
-        <v>24606.84</v>
+        <v>21638.99</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2510,16 +2510,16 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>45662.37361111111</v>
+        <v>45662.37083333333</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>45679.48015942366</v>
+        <v>45678.30954380152</v>
       </c>
       <c r="D62" t="n">
-        <v>24633.43</v>
+        <v>22951.74</v>
       </c>
       <c r="E62" t="n">
-        <v>24609.86</v>
+        <v>22924.32</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -2537,13 +2537,13 @@
         <v>45662.37638888889</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>45679.4842906786</v>
+        <v>45678.37065837454</v>
       </c>
       <c r="D63" t="n">
-        <v>24635.38</v>
+        <v>23031.75</v>
       </c>
       <c r="E63" t="n">
-        <v>24608.39</v>
+        <v>23006.3</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -2558,16 +2558,16 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>45662.35</v>
+        <v>45662.35416666666</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>45679.48824747477</v>
+        <v>45678.38042898908</v>
       </c>
       <c r="D64" t="n">
-        <v>24679.08</v>
+        <v>23077.82</v>
       </c>
       <c r="E64" t="n">
-        <v>24407.38</v>
+        <v>22824.77</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -2582,20 +2582,20 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>45662.37777777778</v>
+        <v>45662.35833333333</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>45679.48845420307</v>
+        <v>45678.48975022274</v>
       </c>
       <c r="D65" t="n">
-        <v>24639.37</v>
+        <v>23229.24</v>
       </c>
       <c r="E65" t="n">
-        <v>24608.73</v>
+        <v>22888.27</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2606,20 +2606,20 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>45662.37916666667</v>
+        <v>45662.36805555555</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>45679.4929093571</v>
+        <v>45679.30275021361</v>
       </c>
       <c r="D66" t="n">
-        <v>24643.79</v>
+        <v>24385.96</v>
       </c>
       <c r="E66" t="n">
-        <v>24613.99</v>
+        <v>23088.95</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2630,20 +2630,20 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>45662.38333333333</v>
+        <v>45662.375</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>45679.49740435466</v>
+        <v>45679.36613700811</v>
       </c>
       <c r="D67" t="n">
-        <v>24644.26</v>
+        <v>24467.24</v>
       </c>
       <c r="E67" t="n">
-        <v>24616.11</v>
+        <v>24203.75</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2654,16 +2654,16 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>45662.38194444445</v>
+        <v>45662.37777777778</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>45679.50081486114</v>
+        <v>45679.45458931023</v>
       </c>
       <c r="D68" t="n">
-        <v>24651.17</v>
+        <v>24590.61</v>
       </c>
       <c r="E68" t="n">
-        <v>24624.37</v>
+        <v>24563.46</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -2678,20 +2678,20 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>45662.36111111111</v>
+        <v>45662.37916666667</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>45680.30615307333</v>
+        <v>45679.45848119786</v>
       </c>
       <c r="D69" t="n">
-        <v>25840.86</v>
+        <v>24594.21</v>
       </c>
       <c r="E69" t="n">
-        <v>24520</v>
+        <v>24564.99</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2702,20 +2702,20 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>45662.38472222222</v>
+        <v>45662.37361111111</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>45680.40084635137</v>
+        <v>45679.46280503023</v>
       </c>
       <c r="D70" t="n">
-        <v>25943.22</v>
+        <v>24608.44</v>
       </c>
       <c r="E70" t="n">
-        <v>25912.95</v>
+        <v>24302.1</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2726,20 +2726,20 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>45662.38611111111</v>
+        <v>45662.38055555556</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>45680.40517113198</v>
+        <v>45679.46295694813</v>
       </c>
       <c r="D71" t="n">
-        <v>25947.45</v>
+        <v>24598.66</v>
       </c>
       <c r="E71" t="n">
-        <v>25921.01</v>
+        <v>23490.82</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2750,20 +2750,20 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>45662.36527777778</v>
+        <v>45662.38194444445</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>45680.40836026006</v>
+        <v>45679.46685187928</v>
       </c>
       <c r="D72" t="n">
-        <v>25982.04</v>
+        <v>24602.27</v>
       </c>
       <c r="E72" t="n">
-        <v>25666.25</v>
+        <v>23498.98</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2774,16 +2774,16 @@
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>45662.3875</v>
+        <v>45662.38333333333</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>45680.40967682941</v>
+        <v>45679.47144544066</v>
       </c>
       <c r="D73" t="n">
-        <v>25951.93</v>
+        <v>24606.88</v>
       </c>
       <c r="E73" t="n">
-        <v>25924.95</v>
+        <v>24577.72</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -2798,20 +2798,20 @@
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>45662.38055555556</v>
+        <v>45662.38611111111</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>45680.5357645696</v>
+        <v>45679.47506898885</v>
       </c>
       <c r="D74" t="n">
-        <v>26143.5</v>
+        <v>24608.1</v>
       </c>
       <c r="E74" t="n">
-        <v>25832.45</v>
+        <v>24577.89</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2822,20 +2822,20 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>45662.375</v>
+        <v>45662.3875</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>45681.29936357489</v>
+        <v>45679.47922680012</v>
       </c>
       <c r="D75" t="n">
-        <v>27251.08</v>
+        <v>24612.09</v>
       </c>
       <c r="E75" t="n">
-        <v>25950.42</v>
+        <v>24585.72</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -2849,13 +2849,13 @@
         <v>45662.38888888889</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>45681.3021171319</v>
+        <v>45679.48314812974</v>
       </c>
       <c r="D76" t="n">
-        <v>27235.05</v>
+        <v>24615.73</v>
       </c>
       <c r="E76" t="n">
-        <v>27208.32</v>
+        <v>24588.25</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -2873,13 +2873,13 @@
         <v>45662.39027777778</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>45681.30630891504</v>
+        <v>45679.48728703719</v>
       </c>
       <c r="D77" t="n">
-        <v>27239.08</v>
+        <v>24619.69</v>
       </c>
       <c r="E77" t="n">
-        <v>27211.24</v>
+        <v>24593.78</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -2897,13 +2897,13 @@
         <v>45662.39166666667</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>45681.30929125974</v>
+        <v>45679.49073334755</v>
       </c>
       <c r="D78" t="n">
-        <v>27241.38</v>
+        <v>24622.66</v>
       </c>
       <c r="E78" t="n">
-        <v>27213.53</v>
+        <v>24601.31</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -2918,16 +2918,16 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>45662.39305555556</v>
+        <v>45662.39583333334</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>45681.31366135218</v>
+        <v>45680.29576971807</v>
       </c>
       <c r="D79" t="n">
-        <v>27245.67</v>
+        <v>25775.91</v>
       </c>
       <c r="E79" t="n">
-        <v>27217.19</v>
+        <v>25749.21</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -2942,16 +2942,16 @@
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>45662.39444444444</v>
+        <v>45662.4</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>45681.31803175672</v>
+        <v>45680.29836126349</v>
       </c>
       <c r="D80" t="n">
-        <v>27249.97</v>
+        <v>25773.64</v>
       </c>
       <c r="E80" t="n">
-        <v>27222.06</v>
+        <v>25747.38</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -2966,16 +2966,16 @@
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>45662.39722222222</v>
+        <v>45662.40138888889</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>45681.3209855744</v>
+        <v>45680.30192706605</v>
       </c>
       <c r="D81" t="n">
-        <v>27250.22</v>
+        <v>25776.77</v>
       </c>
       <c r="E81" t="n">
-        <v>27225.54</v>
+        <v>25747.45</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -2990,16 +2990,16 @@
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>45662.39861111111</v>
+        <v>45662.40416666667</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>45681.3242839368</v>
+        <v>45680.30552237033</v>
       </c>
       <c r="D82" t="n">
-        <v>27252.97</v>
+        <v>25777.95</v>
       </c>
       <c r="E82" t="n">
-        <v>27226.11</v>
+        <v>25754.2</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -3014,20 +3014,20 @@
         </is>
       </c>
       <c r="B83" s="2" t="n">
-        <v>45662.4</v>
+        <v>45662.38472222222</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>45681.32760307437</v>
+        <v>45680.30775151414</v>
       </c>
       <c r="D83" t="n">
-        <v>27255.75</v>
+        <v>25809.16</v>
       </c>
       <c r="E83" t="n">
-        <v>27231.83</v>
+        <v>24537.75</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -3038,16 +3038,16 @@
         </is>
       </c>
       <c r="B84" s="2" t="n">
-        <v>45662.40277777778</v>
+        <v>45662.40694444445</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>45681.33119633021</v>
+        <v>45680.30977670962</v>
       </c>
       <c r="D84" t="n">
-        <v>27256.92</v>
+        <v>25780.08</v>
       </c>
       <c r="E84" t="n">
-        <v>27228.59</v>
+        <v>25751.57</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -3062,16 +3062,16 @@
         </is>
       </c>
       <c r="B85" s="2" t="n">
-        <v>45662.40555555555</v>
+        <v>45662.40833333333</v>
       </c>
       <c r="C85" s="2" t="n">
-        <v>45681.33461168112</v>
+        <v>45680.31349175517</v>
       </c>
       <c r="D85" t="n">
-        <v>27257.84</v>
+        <v>25783.43</v>
       </c>
       <c r="E85" t="n">
-        <v>27235.5</v>
+        <v>25754.58</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -3086,16 +3086,16 @@
         </is>
       </c>
       <c r="B86" s="2" t="n">
-        <v>45662.40416666667</v>
+        <v>45662.40972222222</v>
       </c>
       <c r="C86" s="2" t="n">
-        <v>45681.33846355641</v>
+        <v>45680.31586802262</v>
       </c>
       <c r="D86" t="n">
-        <v>27265.39</v>
+        <v>25784.85</v>
       </c>
       <c r="E86" t="n">
-        <v>27234.89</v>
+        <v>25764.63</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -3110,16 +3110,16 @@
         </is>
       </c>
       <c r="B87" s="2" t="n">
-        <v>45662.40694444445</v>
+        <v>45662.41111111111</v>
       </c>
       <c r="C87" s="2" t="n">
-        <v>45681.34197540774</v>
+        <v>45680.3193618877</v>
       </c>
       <c r="D87" t="n">
-        <v>27266.44</v>
+        <v>25787.88</v>
       </c>
       <c r="E87" t="n">
-        <v>27237.76</v>
+        <v>25761.42</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="B88" s="2" t="n">
-        <v>45662.40833333333</v>
+        <v>45662.4125</v>
       </c>
       <c r="C88" s="2" t="n">
-        <v>45681.34628781332</v>
+        <v>45680.322826858</v>
       </c>
       <c r="D88" t="n">
-        <v>27270.65</v>
+        <v>25790.87</v>
       </c>
       <c r="E88" t="n">
-        <v>27242.27</v>
+        <v>25762.06</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -3158,16 +3158,16 @@
         </is>
       </c>
       <c r="B89" s="2" t="n">
-        <v>45662.40972222222</v>
+        <v>45662.41388888889</v>
       </c>
       <c r="C89" s="2" t="n">
-        <v>45681.34972006597</v>
+        <v>45680.32727616818</v>
       </c>
       <c r="D89" t="n">
-        <v>27273.6</v>
+        <v>25795.28</v>
       </c>
       <c r="E89" t="n">
-        <v>27244.35</v>
+        <v>25767.63</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -3182,16 +3182,16 @@
         </is>
       </c>
       <c r="B90" s="2" t="n">
-        <v>45662.4125</v>
+        <v>45662.41527777778</v>
       </c>
       <c r="C90" s="2" t="n">
-        <v>45681.35353542436</v>
+        <v>45680.33194784635</v>
       </c>
       <c r="D90" t="n">
-        <v>27275.09</v>
+        <v>25800</v>
       </c>
       <c r="E90" t="n">
-        <v>27248.95</v>
+        <v>25773.35</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -3206,16 +3206,16 @@
         </is>
       </c>
       <c r="B91" s="2" t="n">
-        <v>45662.41388888889</v>
+        <v>45662.41666666666</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>45681.35595963308</v>
+        <v>45680.33647128829</v>
       </c>
       <c r="D91" t="n">
-        <v>27276.58</v>
+        <v>25804.52</v>
       </c>
       <c r="E91" t="n">
-        <v>27248.41</v>
+        <v>25779.71</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -3230,20 +3230,20 @@
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>45662.41527777778</v>
+        <v>45662.39444444444</v>
       </c>
       <c r="C92" s="2" t="n">
-        <v>45681.36052819547</v>
+        <v>45680.45165215246</v>
       </c>
       <c r="D92" t="n">
-        <v>27281.16</v>
+        <v>26002.38</v>
       </c>
       <c r="E92" t="n">
-        <v>27254.37</v>
+        <v>25674.61</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -3254,20 +3254,20 @@
         </is>
       </c>
       <c r="B93" s="2" t="n">
-        <v>45662.41111111111</v>
+        <v>45662.39305555556</v>
       </c>
       <c r="C93" s="2" t="n">
-        <v>45682.4118632898</v>
+        <v>45681.30395412225</v>
       </c>
       <c r="D93" t="n">
-        <v>28801.08</v>
+        <v>27231.69</v>
       </c>
       <c r="E93" t="n">
-        <v>28502.08</v>
+        <v>25809.91</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -3278,16 +3278,16 @@
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>45662.41666666666</v>
+        <v>45662.41805555556</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>45682.41508173538</v>
+        <v>45681.4000094676</v>
       </c>
       <c r="D94" t="n">
-        <v>28797.72</v>
+        <v>27334.01</v>
       </c>
       <c r="E94" t="n">
-        <v>28772.41</v>
+        <v>27305.33</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -3302,20 +3302,20 @@
         </is>
       </c>
       <c r="B95" s="2" t="n">
-        <v>45662.41805555556</v>
+        <v>45662.39722222222</v>
       </c>
       <c r="C95" s="2" t="n">
-        <v>45682.41875947017</v>
+        <v>45681.41150844435</v>
       </c>
       <c r="D95" t="n">
-        <v>28801.01</v>
+        <v>27380.57</v>
       </c>
       <c r="E95" t="n">
-        <v>28775.32</v>
+        <v>27061.64</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -3326,20 +3326,20 @@
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>45662.41944444444</v>
+        <v>45662.39861111111</v>
       </c>
       <c r="C96" s="2" t="n">
-        <v>45682.42328160448</v>
+        <v>45681.5152986481</v>
       </c>
       <c r="D96" t="n">
-        <v>28805.53</v>
+        <v>27528.03</v>
       </c>
       <c r="E96" t="n">
-        <v>28777.75</v>
+        <v>27220.58</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -3350,16 +3350,16 @@
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>45662.42361111111</v>
+        <v>45662.41944444444</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>45682.42780392143</v>
+        <v>45682.29557146539</v>
       </c>
       <c r="D97" t="n">
-        <v>28806.04</v>
+        <v>28621.62</v>
       </c>
       <c r="E97" t="n">
-        <v>28781.2</v>
+        <v>28592.06</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -3374,20 +3374,20 @@
         </is>
       </c>
       <c r="B98" s="2" t="n">
-        <v>45662.42222222222</v>
+        <v>45662.40555555555</v>
       </c>
       <c r="C98" s="2" t="n">
-        <v>45682.50846915448</v>
+        <v>45682.30482944068</v>
       </c>
       <c r="D98" t="n">
-        <v>28924.2</v>
+        <v>28654.95</v>
       </c>
       <c r="E98" t="n">
-        <v>27819.88</v>
+        <v>27387.42</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -3398,20 +3398,644 @@
         </is>
       </c>
       <c r="B99" s="2" t="n">
+        <v>45662.42083333333</v>
+      </c>
+      <c r="C99" s="2" t="n">
+        <v>45682.36125961172</v>
+      </c>
+      <c r="D99" t="n">
+        <v>28714.21</v>
+      </c>
+      <c r="E99" t="n">
+        <v>28689.41</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="n">
+        <v>45662.42222222222</v>
+      </c>
+      <c r="C100" s="2" t="n">
+        <v>45682.36506481839</v>
+      </c>
+      <c r="D100" t="n">
+        <v>28717.69</v>
+      </c>
+      <c r="E100" t="n">
+        <v>28688.22</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="n">
+        <v>45662.42361111111</v>
+      </c>
+      <c r="C101" s="2" t="n">
+        <v>45682.36950473118</v>
+      </c>
+      <c r="D101" t="n">
+        <v>28722.09</v>
+      </c>
+      <c r="E101" t="n">
+        <v>28690.55</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="n">
+        <v>45662.40277777778</v>
+      </c>
+      <c r="C102" s="2" t="n">
+        <v>45682.37171391879</v>
+      </c>
+      <c r="D102" t="n">
+        <v>28755.27</v>
+      </c>
+      <c r="E102" t="n">
+        <v>28515.25</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="n">
         <v>45662.425</v>
       </c>
-      <c r="C99" s="2" t="n">
-        <v>45682.511289335</v>
-      </c>
-      <c r="D99" t="n">
-        <v>28924.26</v>
-      </c>
-      <c r="E99" t="n">
-        <v>28903.7</v>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+      <c r="C103" s="2" t="n">
+        <v>45682.37232945213</v>
+      </c>
+      <c r="D103" t="n">
+        <v>28724.15</v>
+      </c>
+      <c r="E103" t="n">
+        <v>28698.87</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="n">
+        <v>45662.42638888889</v>
+      </c>
+      <c r="C104" s="2" t="n">
+        <v>45682.37644474079</v>
+      </c>
+      <c r="D104" t="n">
+        <v>28728.08</v>
+      </c>
+      <c r="E104" t="n">
+        <v>28700.18</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="n">
+        <v>45662.42777777778</v>
+      </c>
+      <c r="C105" s="2" t="n">
+        <v>45682.3806963802</v>
+      </c>
+      <c r="D105" t="n">
+        <v>28732.2</v>
+      </c>
+      <c r="E105" t="n">
+        <v>28704.42</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="n">
+        <v>45662.42916666667</v>
+      </c>
+      <c r="C106" s="2" t="n">
+        <v>45682.38506751259</v>
+      </c>
+      <c r="D106" t="n">
+        <v>28736.5</v>
+      </c>
+      <c r="E106" t="n">
+        <v>28709.36</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="n">
+        <v>45662.43055555555</v>
+      </c>
+      <c r="C107" s="2" t="n">
+        <v>45682.38970902534</v>
+      </c>
+      <c r="D107" t="n">
+        <v>28741.18</v>
+      </c>
+      <c r="E107" t="n">
+        <v>28712.76</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="n">
+        <v>45662.43194444444</v>
+      </c>
+      <c r="C108" s="2" t="n">
+        <v>45682.39383160766</v>
+      </c>
+      <c r="D108" t="n">
+        <v>28745.12</v>
+      </c>
+      <c r="E108" t="n">
+        <v>28715.49</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="n">
+        <v>45662.43333333333</v>
+      </c>
+      <c r="C109" s="2" t="n">
+        <v>45682.39839205483</v>
+      </c>
+      <c r="D109" t="n">
+        <v>28749.68</v>
+      </c>
+      <c r="E109" t="n">
+        <v>28721.07</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="n">
+        <v>45662.43611111111</v>
+      </c>
+      <c r="C110" s="2" t="n">
+        <v>45682.40189128138</v>
+      </c>
+      <c r="D110" t="n">
+        <v>28750.72</v>
+      </c>
+      <c r="E110" t="n">
+        <v>28722.48</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="n">
+        <v>45662.43472222222</v>
+      </c>
+      <c r="C111" s="2" t="n">
+        <v>45682.50878649591</v>
+      </c>
+      <c r="D111" t="n">
+        <v>28906.65</v>
+      </c>
+      <c r="E111" t="n">
+        <v>27638.83</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="n">
+        <v>45662.44027777778</v>
+      </c>
+      <c r="C112" s="2" t="n">
+        <v>45683.29476731822</v>
+      </c>
+      <c r="D112" t="n">
+        <v>30030.46</v>
+      </c>
+      <c r="E112" t="n">
+        <v>30006.79</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="n">
+        <v>45662.44305555556</v>
+      </c>
+      <c r="C113" s="2" t="n">
+        <v>45683.298002282</v>
+      </c>
+      <c r="D113" t="n">
+        <v>30031.12</v>
+      </c>
+      <c r="E113" t="n">
+        <v>30004.98</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="n">
+        <v>45662.44444444445</v>
+      </c>
+      <c r="C114" s="2" t="n">
+        <v>45683.3022160192</v>
+      </c>
+      <c r="D114" t="n">
+        <v>30035.19</v>
+      </c>
+      <c r="E114" t="n">
+        <v>30008.65</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="n">
+        <v>45662.44583333333</v>
+      </c>
+      <c r="C115" s="2" t="n">
+        <v>45683.30569821764</v>
+      </c>
+      <c r="D115" t="n">
+        <v>30038.21</v>
+      </c>
+      <c r="E115" t="n">
+        <v>30012.82</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="n">
+        <v>45662.4375</v>
+      </c>
+      <c r="C116" s="2" t="n">
+        <v>45683.30742214988</v>
+      </c>
+      <c r="D116" t="n">
+        <v>30052.69</v>
+      </c>
+      <c r="E116" t="n">
+        <v>27785.09</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="n">
+        <v>45662.44861111111</v>
+      </c>
+      <c r="C117" s="2" t="n">
+        <v>45683.30945422715</v>
+      </c>
+      <c r="D117" t="n">
+        <v>30039.61</v>
+      </c>
+      <c r="E117" t="n">
+        <v>30014.03</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="n">
+        <v>45662.45277777778</v>
+      </c>
+      <c r="C118" s="2" t="n">
+        <v>45683.31297951594</v>
+      </c>
+      <c r="D118" t="n">
+        <v>30038.69</v>
+      </c>
+      <c r="E118" t="n">
+        <v>30011.46</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="n">
+        <v>45662.45416666667</v>
+      </c>
+      <c r="C119" s="2" t="n">
+        <v>45683.3914549181</v>
+      </c>
+      <c r="D119" t="n">
+        <v>30149.7</v>
+      </c>
+      <c r="E119" t="n">
+        <v>30121.08</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="n">
+        <v>45662.45555555556</v>
+      </c>
+      <c r="C120" s="2" t="n">
+        <v>45683.39545692968</v>
+      </c>
+      <c r="D120" t="n">
+        <v>30153.46</v>
+      </c>
+      <c r="E120" t="n">
+        <v>30129.32</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="n">
+        <v>45662.44166666667</v>
+      </c>
+      <c r="C121" s="2" t="n">
+        <v>45683.40281377276</v>
+      </c>
+      <c r="D121" t="n">
+        <v>30184.05</v>
+      </c>
+      <c r="E121" t="n">
+        <v>29954.72</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="n">
+        <v>45662.44722222222</v>
+      </c>
+      <c r="C122" s="2" t="n">
+        <v>45683.48528964628</v>
+      </c>
+      <c r="D122" t="n">
+        <v>30294.82</v>
+      </c>
+      <c r="E122" t="n">
+        <v>30057.57</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="n">
+        <v>45662.43888888889</v>
+      </c>
+      <c r="C123" s="2" t="n">
+        <v>45683.53375720033</v>
+      </c>
+      <c r="D123" t="n">
+        <v>30376.61</v>
+      </c>
+      <c r="E123" t="n">
+        <v>29038.09</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="n">
+        <v>45662.45138888889</v>
+      </c>
+      <c r="C124" s="2" t="n">
+        <v>45684.30524191434</v>
+      </c>
+      <c r="D124" t="n">
+        <v>31469.55</v>
+      </c>
+      <c r="E124" t="n">
+        <v>30217.91</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="n">
+        <v>45662.45</v>
+      </c>
+      <c r="C125" s="2" t="n">
+        <v>45684.40300360583</v>
+      </c>
+      <c r="D125" t="n">
+        <v>31612.33</v>
+      </c>
+      <c r="E125" t="n">
+        <v>31276.63</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -3458,7 +4082,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>98</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4">
@@ -3468,7 +4092,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>95.65000000000001</v>
+        <v>96.77</v>
       </c>
     </row>
     <row r="5">
@@ -3478,7 +4102,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>9.710000000000001</v>
+        <v>10.36</v>
       </c>
     </row>
     <row r="6">
@@ -3488,7 +4112,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11.81</v>
+        <v>11.85</v>
       </c>
     </row>
     <row r="7">
@@ -3498,7 +4122,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>55.56</v>
+        <v>4.46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactored code now runs.  Need to imporve GUI to include scroll bars.  Also, need to have results include the same format as the Bizagi simulation.  Also, simulation not behaving properly when the number of day to simulate is modified.
</commit_message>
<xml_diff>
--- a/5.5.13 Real Property-Monthly Reviews-2_results.xlsx
+++ b/5.5.13 Real Property-Monthly Reviews-2_results.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.36</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -464,7 +464,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.09</v>
+        <v>18.28</v>
       </c>
     </row>
   </sheetData>
@@ -573,40 +573,40 @@
         <v>500</v>
       </c>
       <c r="D2" t="n">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="E2" t="n">
-        <v>24.8</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>59.95</v>
+        <v>36.79</v>
       </c>
       <c r="G2" t="n">
-        <v>31612.33</v>
+        <v>40128.31</v>
       </c>
       <c r="H2" t="n">
-        <v>18879.43</v>
+        <v>22875.19</v>
       </c>
       <c r="I2" t="n">
-        <v>23077.82</v>
+        <v>24540.37</v>
       </c>
       <c r="J2" t="n">
-        <v>10449.24</v>
+        <v>11370.14</v>
       </c>
       <c r="K2" t="n">
-        <v>30030.93</v>
+        <v>35881.35</v>
       </c>
       <c r="L2" t="n">
-        <v>2304145.7</v>
+        <v>2567094.41</v>
       </c>
       <c r="M2" t="n">
-        <v>32.97</v>
+        <v>24.57</v>
       </c>
       <c r="N2" t="n">
-        <v>31276.63</v>
+        <v>40113.93</v>
       </c>
       <c r="O2" t="n">
-        <v>18581.82</v>
+        <v>22717.65</v>
       </c>
     </row>
     <row r="3">
@@ -672,43 +672,43 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="D4" t="n">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>5.19</v>
+        <v>5.16</v>
       </c>
       <c r="G4" t="n">
         <v>9.58</v>
       </c>
       <c r="H4" t="n">
-        <v>8.1</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>8.24</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>1.04</v>
+        <v>1.05</v>
       </c>
       <c r="K4" t="n">
-        <v>9.35</v>
+        <v>9.34</v>
       </c>
       <c r="L4" t="n">
-        <v>10183752.51</v>
+        <v>6529118.03</v>
       </c>
       <c r="M4" t="n">
-        <v>6.21</v>
+        <v>5.92</v>
       </c>
       <c r="N4" t="n">
-        <v>20332.4</v>
+        <v>29988.34</v>
       </c>
       <c r="O4" t="n">
-        <v>10255.54</v>
+        <v>13084.4</v>
       </c>
     </row>
     <row r="5">
@@ -723,10 +723,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="D5" t="n">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="E5" t="n">
         <v>100</v>
@@ -774,43 +774,43 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="D6" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E6" t="n">
         <v>100</v>
       </c>
       <c r="F6" t="n">
-        <v>3.42</v>
+        <v>3.46</v>
       </c>
       <c r="G6" t="n">
-        <v>6.73</v>
+        <v>6.7</v>
       </c>
       <c r="H6" t="n">
         <v>5.53</v>
       </c>
       <c r="I6" t="n">
-        <v>5.65</v>
+        <v>5.86</v>
       </c>
       <c r="J6" t="n">
-        <v>0.82</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="K6" t="n">
-        <v>6.55</v>
+        <v>6.57</v>
       </c>
       <c r="L6" t="n">
-        <v>3098701.11</v>
+        <v>1750713.92</v>
       </c>
       <c r="M6" t="n">
-        <v>32.97</v>
+        <v>24.57</v>
       </c>
       <c r="N6" t="n">
-        <v>27225.48</v>
+        <v>35840.76</v>
       </c>
       <c r="O6" t="n">
-        <v>16570.59</v>
+        <v>20596.63</v>
       </c>
     </row>
     <row r="7">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="D7" t="n">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="E7" t="n">
         <v>100</v>
@@ -852,16 +852,16 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>8.57</v>
+        <v>1316.14</v>
       </c>
       <c r="M7" t="n">
-        <v>8.57</v>
+        <v>6.31</v>
       </c>
       <c r="N7" t="n">
-        <v>8.57</v>
+        <v>1085.12</v>
       </c>
       <c r="O7" t="n">
-        <v>8.57</v>
+        <v>52.65</v>
       </c>
     </row>
     <row r="8">
@@ -876,43 +876,43 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D8" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E8" t="n">
         <v>100</v>
       </c>
       <c r="F8" t="n">
-        <v>70.27</v>
+        <v>91.65000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>161.49</v>
+        <v>162.38</v>
       </c>
       <c r="H8" t="n">
-        <v>126.06</v>
+        <v>126.69</v>
       </c>
       <c r="I8" t="n">
-        <v>133.75</v>
+        <v>126.08</v>
       </c>
       <c r="J8" t="n">
-        <v>27.1</v>
+        <v>20.31</v>
       </c>
       <c r="K8" t="n">
-        <v>156.43</v>
+        <v>156.88</v>
       </c>
       <c r="L8" t="n">
-        <v>1031770.38</v>
+        <v>512991.15</v>
       </c>
       <c r="M8" t="n">
-        <v>1510.3</v>
+        <v>58.03</v>
       </c>
       <c r="N8" t="n">
-        <v>27125.38</v>
+        <v>31774.25</v>
       </c>
       <c r="O8" t="n">
-        <v>19106.86</v>
+        <v>20519.65</v>
       </c>
     </row>
     <row r="9">
@@ -927,10 +927,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D9" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E9" t="n">
         <v>100</v>
@@ -978,43 +978,43 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D10" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E10" t="n">
-        <v>96.77</v>
+        <v>100</v>
       </c>
       <c r="F10" t="n">
-        <v>7.59</v>
+        <v>6.31</v>
       </c>
       <c r="G10" t="n">
-        <v>12.07</v>
+        <v>11.97</v>
       </c>
       <c r="H10" t="n">
-        <v>10.36</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>10.58</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J10" t="n">
-        <v>1.27</v>
+        <v>1.75</v>
       </c>
       <c r="K10" t="n">
-        <v>11.85</v>
+        <v>11.81</v>
       </c>
       <c r="L10" t="n">
-        <v>129.44</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>6.83</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>4.46</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1028,7 +1028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1066,2976 +1066,2712 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-1</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>45662.29166666666</v>
+        <v>45663.29166666666</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45662.33329752198</v>
+        <v>45663.31721341277</v>
       </c>
       <c r="D2" t="n">
-        <v>59.95</v>
+        <v>36.79</v>
       </c>
       <c r="E2" t="n">
-        <v>32.97</v>
+        <v>24.57</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-2</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>45662.29305555556</v>
+        <v>45663.29305555556</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>45662.37334402597</v>
+        <v>45663.43960284361</v>
       </c>
       <c r="D3" t="n">
-        <v>115.62</v>
+        <v>211.03</v>
       </c>
       <c r="E3" t="n">
-        <v>87.23</v>
+        <v>71.36</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-3</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>45662.29583333333</v>
+        <v>45663.29444444444</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>45662.40163947275</v>
+        <v>45664.2971430707</v>
       </c>
       <c r="D4" t="n">
-        <v>152.36</v>
+        <v>1443.89</v>
       </c>
       <c r="E4" t="n">
-        <v>125.87</v>
+        <v>239.9</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-4</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>45662.29722222222</v>
+        <v>45663.29583333333</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>45662.43762263396</v>
+        <v>45664.31772866953</v>
       </c>
       <c r="D5" t="n">
-        <v>202.18</v>
+        <v>1471.53</v>
       </c>
       <c r="E5" t="n">
-        <v>179.17</v>
+        <v>1457.31</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-5</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>45662.29861111111</v>
+        <v>45663.29722222222</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>45662.46990041722</v>
+        <v>45664.3554593779</v>
       </c>
       <c r="D6" t="n">
-        <v>246.66</v>
+        <v>1523.86</v>
       </c>
       <c r="E6" t="n">
-        <v>219.67</v>
+        <v>1510.88</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-6</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>45662.3</v>
+        <v>45663.29861111111</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>45662.51885033459</v>
+        <v>45664.38601615631</v>
       </c>
       <c r="D7" t="n">
-        <v>315.14</v>
+        <v>1565.86</v>
       </c>
       <c r="E7" t="n">
-        <v>285.13</v>
+        <v>1550.43</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-7</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>45662.30138888889</v>
+        <v>45663.3</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>45662.5399183164</v>
+        <v>45664.41771524574</v>
       </c>
       <c r="D8" t="n">
-        <v>343.48</v>
+        <v>1609.51</v>
       </c>
       <c r="E8" t="n">
-        <v>316.25</v>
+        <v>1593.42</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-8</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>45662.30277777778</v>
+        <v>45663.30138888889</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>45663.31580679751</v>
+        <v>45664.51319002151</v>
       </c>
       <c r="D9" t="n">
-        <v>1458.76</v>
+        <v>1744.99</v>
       </c>
       <c r="E9" t="n">
-        <v>1431.38</v>
+        <v>1642.04</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-103</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>45662.30416666667</v>
+        <v>45663.43333333333</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45663.35101653879</v>
+        <v>45666.37843254983</v>
       </c>
       <c r="D10" t="n">
-        <v>1507.46</v>
+        <v>4240.94</v>
       </c>
       <c r="E10" t="n">
-        <v>1480.52</v>
+        <v>4227.79</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-9</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>45662.30555555555</v>
+        <v>45663.30277777778</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>45663.39079347986</v>
+        <v>45666.40604065492</v>
       </c>
       <c r="D11" t="n">
-        <v>1562.74</v>
+        <v>4468.7</v>
       </c>
       <c r="E11" t="n">
-        <v>1532.57</v>
+        <v>4455.27</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-10</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45662.30833333333</v>
+        <v>45663.30416666667</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>45663.43154756449</v>
+        <v>45667.29166666666</v>
       </c>
       <c r="D12" t="n">
-        <v>1617.43</v>
+        <v>5742</v>
       </c>
       <c r="E12" t="n">
-        <v>1589.82</v>
+        <v>5573.6</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-11</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>45662.29444444444</v>
+        <v>45663.30555555555</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>45663.5338707749</v>
+        <v>45667.31224586003</v>
       </c>
       <c r="D13" t="n">
-        <v>1784.77</v>
+        <v>5769.63</v>
       </c>
       <c r="E13" t="n">
-        <v>1532.25</v>
+        <v>5757.25</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-12</t>
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>45662.31111111111</v>
+        <v>45663.30694444444</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>45664.3203193547</v>
+        <v>45667.33770677419</v>
       </c>
       <c r="D14" t="n">
-        <v>2893.26</v>
+        <v>5804.3</v>
       </c>
       <c r="E14" t="n">
-        <v>2864.74</v>
+        <v>5791.23</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-13</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>45662.3125</v>
+        <v>45663.30833333333</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>45664.34962421956</v>
+        <v>45667.36589191009</v>
       </c>
       <c r="D15" t="n">
-        <v>2933.46</v>
+        <v>5842.88</v>
       </c>
       <c r="E15" t="n">
-        <v>2907.38</v>
+        <v>5827.73</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-181</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>45662.31527777778</v>
+        <v>45664.29166666666</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>45664.41355094349</v>
+        <v>45670.44068827211</v>
       </c>
       <c r="D16" t="n">
-        <v>3021.51</v>
+        <v>8854.59</v>
       </c>
       <c r="E16" t="n">
-        <v>2990.55</v>
+        <v>8839.190000000001</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-14</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>45662.31666666667</v>
+        <v>45663.30972222222</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>45664.43969734229</v>
+        <v>45670.46319867545</v>
       </c>
       <c r="D17" t="n">
-        <v>3057.16</v>
+        <v>10301.01</v>
       </c>
       <c r="E17" t="n">
-        <v>3029.78</v>
+        <v>10288.28</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-15</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>45662.31805555556</v>
+        <v>45663.31111111111</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>45664.46696351265</v>
+        <v>45671.29768164405</v>
       </c>
       <c r="D18" t="n">
-        <v>3094.43</v>
+        <v>11500.66</v>
       </c>
       <c r="E18" t="n">
-        <v>3065.71</v>
+        <v>10330.58</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-16</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>45662.32222222222</v>
+        <v>45663.3125</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>45665.30706725767</v>
+        <v>45671.31761670134</v>
       </c>
       <c r="D19" t="n">
-        <v>4298.18</v>
+        <v>11527.37</v>
       </c>
       <c r="E19" t="n">
-        <v>4270.89</v>
+        <v>11514.26</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-17</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>45662.32361111111</v>
+        <v>45663.31388888889</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>45665.33880627694</v>
+        <v>45671.34073293558</v>
       </c>
       <c r="D20" t="n">
-        <v>4341.88</v>
+        <v>11558.66</v>
       </c>
       <c r="E20" t="n">
-        <v>4312.75</v>
+        <v>11545.99</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-18</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>45662.325</v>
+        <v>45663.31527777778</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>45665.36845109234</v>
+        <v>45671.38452700573</v>
       </c>
       <c r="D21" t="n">
-        <v>4382.57</v>
+        <v>11619.72</v>
       </c>
       <c r="E21" t="n">
-        <v>4353.12</v>
+        <v>11605.45</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-19</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>45662.31388888889</v>
+        <v>45663.31666666667</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>45665.49950817604</v>
+        <v>45671.41943317295</v>
       </c>
       <c r="D22" t="n">
-        <v>4587.29</v>
+        <v>11667.98</v>
       </c>
       <c r="E22" t="n">
-        <v>4318.61</v>
+        <v>11652.76</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-20</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>45662.30694444444</v>
+        <v>45663.31805555556</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>45666.30669177544</v>
+        <v>45671.43897879779</v>
       </c>
       <c r="D23" t="n">
-        <v>5759.64</v>
+        <v>11694.13</v>
       </c>
       <c r="E23" t="n">
-        <v>4419.3</v>
+        <v>11682.02</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-21</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>45662.32777777778</v>
+        <v>45663.31944444445</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>45666.31027586611</v>
+        <v>45671.46540720287</v>
       </c>
       <c r="D24" t="n">
-        <v>5734.8</v>
+        <v>11730.19</v>
       </c>
       <c r="E24" t="n">
-        <v>5711.16</v>
+        <v>11717.79</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-22</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>45662.32638888889</v>
+        <v>45663.32083333333</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>45666.33877452159</v>
+        <v>45672.29859885221</v>
       </c>
       <c r="D25" t="n">
-        <v>5777.84</v>
+        <v>12927.98</v>
       </c>
       <c r="E25" t="n">
-        <v>5749.81</v>
+        <v>11769.95</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-23</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>45662.32916666667</v>
+        <v>45663.32222222222</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>45666.3760189571</v>
+        <v>45672.31661976408</v>
       </c>
       <c r="D26" t="n">
-        <v>5827.47</v>
+        <v>12951.93</v>
       </c>
       <c r="E26" t="n">
-        <v>5797.79</v>
+        <v>12936.38</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-24</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>45662.33194444444</v>
+        <v>45663.32361111111</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>45666.39543306366</v>
+        <v>45672.36051535398</v>
       </c>
       <c r="D27" t="n">
-        <v>5851.42</v>
+        <v>13013.14</v>
       </c>
       <c r="E27" t="n">
-        <v>5825.24</v>
+        <v>13000.27</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-25</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>45662.33055555556</v>
+        <v>45663.325</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>45666.4291758629</v>
+        <v>45672.38082167129</v>
       </c>
       <c r="D28" t="n">
-        <v>5902.01</v>
+        <v>13040.38</v>
       </c>
       <c r="E28" t="n">
-        <v>5873.09</v>
+        <v>13027.22</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-26</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>45662.33333333334</v>
+        <v>45663.32638888889</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>45666.44954801867</v>
+        <v>45672.40704021512</v>
       </c>
       <c r="D29" t="n">
-        <v>5927.35</v>
+        <v>13076.14</v>
       </c>
       <c r="E29" t="n">
-        <v>5901.38</v>
+        <v>13065.1</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-27</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>45662.30972222222</v>
+        <v>45663.32777777778</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>45667.30633220963</v>
+        <v>45672.43373454718</v>
       </c>
       <c r="D30" t="n">
-        <v>7195.12</v>
+        <v>13112.58</v>
       </c>
       <c r="E30" t="n">
-        <v>5796.98</v>
+        <v>13097.99</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-28</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>45662.48888888889</v>
+        <v>45663.32916666667</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>45667.37023438902</v>
+        <v>45672.45489404738</v>
       </c>
       <c r="D31" t="n">
-        <v>7029.14</v>
+        <v>13141.05</v>
       </c>
       <c r="E31" t="n">
-        <v>5687.5</v>
+        <v>13128.89</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-29</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>45662.32083333333</v>
+        <v>45663.33055555556</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>45667.47586051536</v>
+        <v>45672.50437229722</v>
       </c>
       <c r="D32" t="n">
-        <v>7423.24</v>
+        <v>13210.3</v>
       </c>
       <c r="E32" t="n">
-        <v>7158.56</v>
+        <v>13195.03</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-30</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>45662.33611111111</v>
+        <v>45663.33194444444</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>45667.48772982143</v>
+        <v>45672.53300122751</v>
       </c>
       <c r="D33" t="n">
-        <v>7418.33</v>
+        <v>13249.52</v>
       </c>
       <c r="E33" t="n">
-        <v>7389.91</v>
+        <v>13236.18</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-31</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>45662.3375</v>
+        <v>45663.33333333334</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>45667.52647083604</v>
+        <v>45673.38205540463</v>
       </c>
       <c r="D34" t="n">
-        <v>7472.12</v>
+        <v>14470.16</v>
       </c>
       <c r="E34" t="n">
-        <v>7444.75</v>
+        <v>14353.37</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-32</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>45662.34027777778</v>
+        <v>45663.33472222222</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>45668.41375448016</v>
+        <v>45673.40792404069</v>
       </c>
       <c r="D35" t="n">
-        <v>8745.809999999999</v>
+        <v>14505.41</v>
       </c>
       <c r="E35" t="n">
-        <v>8720.639999999999</v>
+        <v>14490.48</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-33</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>45662.31944444445</v>
+        <v>45663.33611111111</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>45668.41976485375</v>
+        <v>45673.51901447696</v>
       </c>
       <c r="D36" t="n">
-        <v>8784.459999999999</v>
+        <v>14663.38</v>
       </c>
       <c r="E36" t="n">
-        <v>8457.84</v>
+        <v>14533.5</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-34</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>45662.33888888889</v>
+        <v>45663.3375</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>45668.44414685827</v>
+        <v>45674.295780187</v>
       </c>
       <c r="D37" t="n">
-        <v>8791.57</v>
+        <v>15779.92</v>
       </c>
       <c r="E37" t="n">
-        <v>8764.33</v>
+        <v>15766.5</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-35</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>45662.34166666667</v>
+        <v>45663.33888888889</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>45668.4639501508</v>
+        <v>45674.32342070774</v>
       </c>
       <c r="D38" t="n">
-        <v>8816.09</v>
+        <v>15817.73</v>
       </c>
       <c r="E38" t="n">
-        <v>8794.24</v>
+        <v>15803.71</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-36</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>45662.34305555555</v>
+        <v>45663.34027777778</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>45668.50091386359</v>
+        <v>45674.35048978139</v>
       </c>
       <c r="D39" t="n">
-        <v>8867.32</v>
+        <v>15854.71</v>
       </c>
       <c r="E39" t="n">
-        <v>8841.049999999999</v>
+        <v>15839.6</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-37</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>45662.33472222222</v>
+        <v>45663.34166666667</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>45669.30678219995</v>
+        <v>45674.38200978176</v>
       </c>
       <c r="D40" t="n">
-        <v>10039.77</v>
+        <v>15898.09</v>
       </c>
       <c r="E40" t="n">
-        <v>7766.26</v>
+        <v>15883.09</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-335</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>45662.34444444445</v>
+        <v>45664.50555555556</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>45669.53506792918</v>
+        <v>45677.39655038607</v>
       </c>
       <c r="D41" t="n">
-        <v>10354.5</v>
+        <v>18563.03</v>
       </c>
       <c r="E41" t="n">
-        <v>9250.26</v>
+        <v>18547.43</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-38</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>45662.85138888889</v>
+        <v>45663.34305555555</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>45670.41012530989</v>
+        <v>45677.42384014429</v>
       </c>
       <c r="D42" t="n">
-        <v>10884.58</v>
+        <v>20276.33</v>
       </c>
       <c r="E42" t="n">
-        <v>8970.440000000001</v>
+        <v>20263.99</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-39</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>45662.69305555556</v>
+        <v>45663.34444444445</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>45674.41309944067</v>
+        <v>45677.44931287152</v>
       </c>
       <c r="D43" t="n">
-        <v>16876.86</v>
+        <v>20311.01</v>
       </c>
       <c r="E43" t="n">
-        <v>14727.07</v>
+        <v>20298.97</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-40</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>45662.88472222222</v>
+        <v>45663.34583333333</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>45675.41094876696</v>
+        <v>45677.47497442387</v>
       </c>
       <c r="D44" t="n">
-        <v>18037.77</v>
+        <v>20345.96</v>
       </c>
       <c r="E44" t="n">
-        <v>16140.3</v>
+        <v>20335.46</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-41</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>45662.83333333334</v>
+        <v>45663.34722222222</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>45677.36096354036</v>
+        <v>45677.50290023257</v>
       </c>
       <c r="D45" t="n">
-        <v>20919.79</v>
+        <v>20384.18</v>
       </c>
       <c r="E45" t="n">
-        <v>19061.21</v>
+        <v>20369.65</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-42</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>45662.34722222222</v>
+        <v>45663.34861111111</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>45677.42750575664</v>
+        <v>45678.29806088944</v>
       </c>
       <c r="D46" t="n">
-        <v>21715.61</v>
+        <v>21527.21</v>
       </c>
       <c r="E46" t="n">
-        <v>21688.09</v>
+        <v>20412.05</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-43</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>45662.34861111111</v>
+        <v>45663.35</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>45677.43048310962</v>
+        <v>45678.32033430828</v>
       </c>
       <c r="D47" t="n">
-        <v>21717.9</v>
+        <v>21557.28</v>
       </c>
       <c r="E47" t="n">
-        <v>21691.41</v>
+        <v>21542.9</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-44</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>45662.35</v>
+        <v>45663.35138888889</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>45677.43410099015</v>
+        <v>45678.33959309206</v>
       </c>
       <c r="D48" t="n">
-        <v>21721.11</v>
+        <v>21583.01</v>
       </c>
       <c r="E48" t="n">
-        <v>21695.68</v>
+        <v>20492.94</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-45</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>45662.35138888889</v>
+        <v>45663.35277777778</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>45677.43877493078</v>
+        <v>45678.36494839615</v>
       </c>
       <c r="D49" t="n">
-        <v>21725.84</v>
+        <v>21617.53</v>
       </c>
       <c r="E49" t="n">
-        <v>21696.42</v>
+        <v>21603.65</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-46</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>45662.35277777778</v>
+        <v>45663.35416666666</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>45677.44257253456</v>
+        <v>45678.47365094475</v>
       </c>
       <c r="D50" t="n">
-        <v>21729.3</v>
+        <v>21772.06</v>
       </c>
       <c r="E50" t="n">
-        <v>21703.32</v>
+        <v>21644.66</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-47</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>45662.35555555556</v>
+        <v>45663.35555555556</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>45677.44671235355</v>
+        <v>45678.50031963876</v>
       </c>
       <c r="D51" t="n">
-        <v>21731.27</v>
+        <v>21808.46</v>
       </c>
       <c r="E51" t="n">
-        <v>21705.91</v>
+        <v>21792.52</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-48</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>45662.35694444444</v>
+        <v>45663.35694444444</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>45677.44981649565</v>
+        <v>45678.52839636653</v>
       </c>
       <c r="D52" t="n">
-        <v>21733.74</v>
+        <v>21846.89</v>
       </c>
       <c r="E52" t="n">
-        <v>21706.66</v>
+        <v>21832.74</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-49</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>45662.35972222222</v>
+        <v>45663.35833333333</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>45677.45390445285</v>
+        <v>45679.30709659647</v>
       </c>
       <c r="D53" t="n">
-        <v>21735.62</v>
+        <v>22966.22</v>
       </c>
       <c r="E53" t="n">
-        <v>21707.87</v>
+        <v>22950.99</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-50</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>45662.36111111111</v>
+        <v>45663.35972222222</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>45677.45685047198</v>
+        <v>45679.43205396359</v>
       </c>
       <c r="D54" t="n">
-        <v>21737.86</v>
+        <v>23144.16</v>
       </c>
       <c r="E54" t="n">
-        <v>21711.54</v>
+        <v>22993.06</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-51</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>45662.3625</v>
+        <v>45663.36111111111</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>45677.4611666516</v>
+        <v>45679.45217130476</v>
       </c>
       <c r="D55" t="n">
-        <v>21742.08</v>
+        <v>23171.13</v>
       </c>
       <c r="E55" t="n">
-        <v>21717.84</v>
+        <v>23158.49</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-52</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>45662.36388888889</v>
+        <v>45663.3625</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>45677.4657679312</v>
+        <v>45679.47937049558</v>
       </c>
       <c r="D56" t="n">
-        <v>21746.71</v>
+        <v>23208.29</v>
       </c>
       <c r="E56" t="n">
-        <v>21719.51</v>
+        <v>23192.82</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-53</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>45662.36527777778</v>
+        <v>45663.36388888889</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>45677.46909221537</v>
+        <v>45679.51430672187</v>
       </c>
       <c r="D57" t="n">
-        <v>21749.49</v>
+        <v>23256.6</v>
       </c>
       <c r="E57" t="n">
-        <v>21721.29</v>
+        <v>23241.11</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-54</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>45662.36666666667</v>
+        <v>45663.36527777778</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>45678.29604698024</v>
+        <v>45680.40719872994</v>
       </c>
       <c r="D58" t="n">
-        <v>22938.31</v>
+        <v>24540.37</v>
       </c>
       <c r="E58" t="n">
-        <v>22909.59</v>
+        <v>24372.35</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-55</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>45662.36944444444</v>
+        <v>45663.36666666667</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>45678.30023809815</v>
+        <v>45680.42812662325</v>
       </c>
       <c r="D59" t="n">
-        <v>22940.34</v>
+        <v>24568.5</v>
       </c>
       <c r="E59" t="n">
-        <v>22910.68</v>
+        <v>24554.18</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-56</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>45662.37222222222</v>
+        <v>45663.36805555555</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>45678.30489852621</v>
+        <v>45680.45456403479</v>
       </c>
       <c r="D60" t="n">
-        <v>22943.05</v>
+        <v>24604.57</v>
       </c>
       <c r="E60" t="n">
-        <v>22915.49</v>
+        <v>24591.67</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-57</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>45662.34583333333</v>
+        <v>45663.36944444444</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>45678.30506665447</v>
+        <v>45680.48123043847</v>
       </c>
       <c r="D61" t="n">
-        <v>22981.3</v>
+        <v>24640.97</v>
       </c>
       <c r="E61" t="n">
-        <v>21638.99</v>
+        <v>24628.03</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-58</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>45662.37083333333</v>
+        <v>45663.37083333333</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>45678.30954380152</v>
+        <v>45680.50809453303</v>
       </c>
       <c r="D62" t="n">
-        <v>22951.74</v>
+        <v>24677.66</v>
       </c>
       <c r="E62" t="n">
-        <v>22924.32</v>
+        <v>24664.13</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-59</t>
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>45662.37638888889</v>
+        <v>45663.37222222222</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>45678.37065837454</v>
+        <v>45680.53992029219</v>
       </c>
       <c r="D63" t="n">
-        <v>23031.75</v>
+        <v>24721.49</v>
       </c>
       <c r="E63" t="n">
-        <v>23006.3</v>
+        <v>24706.53</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-60</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>45662.35416666666</v>
+        <v>45663.37361111111</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>45678.38042898908</v>
+        <v>45681.3109905868</v>
       </c>
       <c r="D64" t="n">
-        <v>23077.82</v>
+        <v>25829.83</v>
       </c>
       <c r="E64" t="n">
-        <v>22824.77</v>
+        <v>25814.99</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-61</t>
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>45662.35833333333</v>
+        <v>45663.375</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>45678.48975022274</v>
+        <v>45681.42196762541</v>
       </c>
       <c r="D65" t="n">
-        <v>23229.24</v>
+        <v>25987.63</v>
       </c>
       <c r="E65" t="n">
-        <v>22888.27</v>
+        <v>25869.35</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-62</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>45662.36805555555</v>
+        <v>45663.37638888889</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>45679.30275021361</v>
+        <v>45681.440715653</v>
       </c>
       <c r="D66" t="n">
-        <v>24385.96</v>
+        <v>26012.63</v>
       </c>
       <c r="E66" t="n">
-        <v>23088.95</v>
+        <v>26000.21</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-63</t>
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>45662.375</v>
+        <v>45663.37777777778</v>
       </c>
       <c r="C67" s="2" t="n">
-        <v>45679.36613700811</v>
+        <v>45681.46127413044</v>
       </c>
       <c r="D67" t="n">
-        <v>24467.24</v>
+        <v>26040.23</v>
       </c>
       <c r="E67" t="n">
-        <v>24203.75</v>
+        <v>26029.14</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-64</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>45662.37777777778</v>
+        <v>45663.37916666667</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>45679.45458931023</v>
+        <v>45681.48730194178</v>
       </c>
       <c r="D68" t="n">
-        <v>24590.61</v>
+        <v>26075.71</v>
       </c>
       <c r="E68" t="n">
-        <v>24563.46</v>
+        <v>26063.38</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-65</t>
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>45662.37916666667</v>
+        <v>45663.38055555556</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>45679.45848119786</v>
+        <v>45681.51367038951</v>
       </c>
       <c r="D69" t="n">
-        <v>24594.21</v>
+        <v>26111.69</v>
       </c>
       <c r="E69" t="n">
-        <v>24564.99</v>
+        <v>26101.68</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-66</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>45662.37361111111</v>
+        <v>45663.38194444445</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>45679.46280503023</v>
+        <v>45681.53963501861</v>
       </c>
       <c r="D70" t="n">
-        <v>24608.44</v>
+        <v>26147.07</v>
       </c>
       <c r="E70" t="n">
-        <v>24302.1</v>
+        <v>26132.46</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-67</t>
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>45662.38055555556</v>
+        <v>45663.38333333333</v>
       </c>
       <c r="C71" s="2" t="n">
-        <v>45679.46295694813</v>
+        <v>45684.31340396492</v>
       </c>
       <c r="D71" t="n">
-        <v>24598.66</v>
+        <v>30139.3</v>
       </c>
       <c r="E71" t="n">
-        <v>23490.82</v>
+        <v>30125.07</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-68</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>45662.38194444445</v>
+        <v>45663.38472222222</v>
       </c>
       <c r="C72" s="2" t="n">
-        <v>45679.46685187928</v>
+        <v>45684.42820267653</v>
       </c>
       <c r="D72" t="n">
-        <v>24602.27</v>
+        <v>30302.61</v>
       </c>
       <c r="E72" t="n">
-        <v>23498.98</v>
+        <v>30183.28</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-69</t>
         </is>
       </c>
       <c r="B73" s="2" t="n">
-        <v>45662.38333333333</v>
+        <v>45663.38611111111</v>
       </c>
       <c r="C73" s="2" t="n">
-        <v>45679.47144544066</v>
+        <v>45684.44867335471</v>
       </c>
       <c r="D73" t="n">
-        <v>24606.88</v>
+        <v>30330.09</v>
       </c>
       <c r="E73" t="n">
-        <v>24577.72</v>
+        <v>30314.97</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-70</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>45662.38611111111</v>
+        <v>45663.3875</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>45679.47506898885</v>
+        <v>45685.29747402589</v>
       </c>
       <c r="D74" t="n">
-        <v>24608.1</v>
+        <v>31550.36</v>
       </c>
       <c r="E74" t="n">
-        <v>24577.89</v>
+        <v>30363.88</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-71</t>
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>45662.3875</v>
+        <v>45663.38888888889</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>45679.47922680012</v>
+        <v>45685.42074876856</v>
       </c>
       <c r="D75" t="n">
-        <v>24612.09</v>
+        <v>31725.88</v>
       </c>
       <c r="E75" t="n">
-        <v>24585.72</v>
+        <v>31585.65</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-72</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>45662.38888888889</v>
+        <v>45663.39027777778</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>45679.48314812974</v>
+        <v>45685.4397684663</v>
       </c>
       <c r="D76" t="n">
-        <v>24615.73</v>
+        <v>31751.27</v>
       </c>
       <c r="E76" t="n">
-        <v>24588.25</v>
+        <v>31736.5</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-73</t>
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>45662.39027777778</v>
+        <v>45663.39166666667</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>45679.48728703719</v>
+        <v>45685.46452595351</v>
       </c>
       <c r="D77" t="n">
-        <v>24619.69</v>
+        <v>31784.92</v>
       </c>
       <c r="E77" t="n">
-        <v>24593.78</v>
+        <v>31770.81</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-74</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>45662.39166666667</v>
+        <v>45663.39305555556</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>45679.49073334755</v>
+        <v>45685.49106106194</v>
       </c>
       <c r="D78" t="n">
-        <v>24622.66</v>
+        <v>31821.13</v>
       </c>
       <c r="E78" t="n">
-        <v>24601.31</v>
+        <v>31807.06</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-75</t>
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>45662.39583333334</v>
+        <v>45663.39444444444</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>45680.29576971807</v>
+        <v>45685.51822108388</v>
       </c>
       <c r="D79" t="n">
-        <v>25775.91</v>
+        <v>31858.24</v>
       </c>
       <c r="E79" t="n">
-        <v>25749.21</v>
+        <v>31843.68</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-76</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>45662.4</v>
+        <v>45663.39583333334</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>45680.29836126349</v>
+        <v>45685.5391063725</v>
       </c>
       <c r="D80" t="n">
-        <v>25773.64</v>
+        <v>31886.31</v>
       </c>
       <c r="E80" t="n">
-        <v>25747.38</v>
+        <v>31875.13</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-77</t>
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>45662.40138888889</v>
+        <v>45663.39722222222</v>
       </c>
       <c r="C81" s="2" t="n">
-        <v>45680.30192706605</v>
+        <v>45686.30411175941</v>
       </c>
       <c r="D81" t="n">
-        <v>25776.77</v>
+        <v>32985.92</v>
       </c>
       <c r="E81" t="n">
-        <v>25747.45</v>
+        <v>32974.68</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-78</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>45662.40416666667</v>
+        <v>45663.39861111111</v>
       </c>
       <c r="C82" s="2" t="n">
-        <v>45680.30552237033</v>
+        <v>45686.31916266631</v>
       </c>
       <c r="D82" t="n">
-        <v>25777.95</v>
+        <v>33005.59</v>
       </c>
       <c r="E82" t="n">
-        <v>25754.2</v>
+        <v>32991.52</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-79</t>
         </is>
       </c>
       <c r="B83" s="2" t="n">
-        <v>45662.38472222222</v>
+        <v>45663.4</v>
       </c>
       <c r="C83" s="2" t="n">
-        <v>45680.30775151414</v>
+        <v>45686.43375581441</v>
       </c>
       <c r="D83" t="n">
-        <v>25809.16</v>
+        <v>33168.61</v>
       </c>
       <c r="E83" t="n">
-        <v>24537.75</v>
+        <v>33007.07</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-81</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
-        <v>45662.40694444445</v>
+        <v>45663.40277777778</v>
       </c>
       <c r="C84" s="2" t="n">
-        <v>45680.30977670962</v>
+        <v>45686.50867557069</v>
       </c>
       <c r="D84" t="n">
-        <v>25780.08</v>
+        <v>33272.49</v>
       </c>
       <c r="E84" t="n">
-        <v>25751.57</v>
+        <v>33259.78</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-82</t>
         </is>
       </c>
       <c r="B85" s="2" t="n">
-        <v>45662.40833333333</v>
+        <v>45663.40416666667</v>
       </c>
       <c r="C85" s="2" t="n">
-        <v>45680.31349175517</v>
+        <v>45686.51292416641</v>
       </c>
       <c r="D85" t="n">
-        <v>25783.43</v>
+        <v>33276.61</v>
       </c>
       <c r="E85" t="n">
-        <v>25754.58</v>
+        <v>33261.12</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-80</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
-        <v>45662.40972222222</v>
+        <v>45663.40138888889</v>
       </c>
       <c r="C86" s="2" t="n">
-        <v>45680.31586802262</v>
+        <v>45686.51377314926</v>
       </c>
       <c r="D86" t="n">
-        <v>25784.85</v>
+        <v>33281.83</v>
       </c>
       <c r="E86" t="n">
-        <v>25764.63</v>
+        <v>33160.59</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-83</t>
         </is>
       </c>
       <c r="B87" s="2" t="n">
-        <v>45662.41111111111</v>
+        <v>45663.40555555555</v>
       </c>
       <c r="C87" s="2" t="n">
-        <v>45680.3193618877</v>
+        <v>45686.51691270489</v>
       </c>
       <c r="D87" t="n">
-        <v>25787.88</v>
+        <v>33280.35</v>
       </c>
       <c r="E87" t="n">
-        <v>25761.42</v>
+        <v>33268.39</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-85</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
-        <v>45662.4125</v>
+        <v>45663.40833333333</v>
       </c>
       <c r="C88" s="2" t="n">
-        <v>45680.322826858</v>
+        <v>45687.29479495523</v>
       </c>
       <c r="D88" t="n">
-        <v>25790.87</v>
+        <v>34396.5</v>
       </c>
       <c r="E88" t="n">
-        <v>25762.06</v>
+        <v>34382.62</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-86</t>
         </is>
       </c>
       <c r="B89" s="2" t="n">
-        <v>45662.41388888889</v>
+        <v>45663.40972222222</v>
       </c>
       <c r="C89" s="2" t="n">
-        <v>45680.32727616818</v>
+        <v>45687.29866318146</v>
       </c>
       <c r="D89" t="n">
-        <v>25795.28</v>
+        <v>34400.07</v>
       </c>
       <c r="E89" t="n">
-        <v>25767.63</v>
+        <v>34385.9</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-84</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
-        <v>45662.41527777778</v>
+        <v>45663.40694444445</v>
       </c>
       <c r="C90" s="2" t="n">
-        <v>45680.33194784635</v>
+        <v>45687.29938532144</v>
       </c>
       <c r="D90" t="n">
-        <v>25800</v>
+        <v>34405.11</v>
       </c>
       <c r="E90" t="n">
-        <v>25773.35</v>
+        <v>33280.45</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-87</t>
         </is>
       </c>
       <c r="B91" s="2" t="n">
-        <v>45662.41666666666</v>
+        <v>45663.41111111111</v>
       </c>
       <c r="C91" s="2" t="n">
-        <v>45680.33647128829</v>
+        <v>45687.30274825758</v>
       </c>
       <c r="D91" t="n">
-        <v>25804.52</v>
+        <v>34403.96</v>
       </c>
       <c r="E91" t="n">
-        <v>25779.71</v>
+        <v>34391.38</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-88</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>45662.39444444444</v>
+        <v>45663.4125</v>
       </c>
       <c r="C92" s="2" t="n">
-        <v>45680.45165215246</v>
+        <v>45687.30631757227</v>
       </c>
       <c r="D92" t="n">
-        <v>26002.38</v>
+        <v>34407.1</v>
       </c>
       <c r="E92" t="n">
-        <v>25674.61</v>
+        <v>33317.69</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-89</t>
         </is>
       </c>
       <c r="B93" s="2" t="n">
-        <v>45662.39305555556</v>
+        <v>45663.41388888889</v>
       </c>
       <c r="C93" s="2" t="n">
-        <v>45681.30395412225</v>
+        <v>45687.30961647203</v>
       </c>
       <c r="D93" t="n">
-        <v>27231.69</v>
+        <v>34409.85</v>
       </c>
       <c r="E93" t="n">
-        <v>25809.91</v>
+        <v>34397.41</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-90</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
-        <v>45662.41805555556</v>
+        <v>45663.41527777778</v>
       </c>
       <c r="C94" s="2" t="n">
-        <v>45681.4000094676</v>
+        <v>45687.31401063727</v>
       </c>
       <c r="D94" t="n">
-        <v>27334.01</v>
+        <v>34414.18</v>
       </c>
       <c r="E94" t="n">
-        <v>27305.33</v>
+        <v>34398.83</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-91</t>
         </is>
       </c>
       <c r="B95" s="2" t="n">
-        <v>45662.39722222222</v>
+        <v>45663.41666666666</v>
       </c>
       <c r="C95" s="2" t="n">
-        <v>45681.41150844435</v>
+        <v>45687.31862709111</v>
       </c>
       <c r="D95" t="n">
-        <v>27380.57</v>
+        <v>34418.82</v>
       </c>
       <c r="E95" t="n">
-        <v>27061.64</v>
+        <v>34402.86</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-92</t>
         </is>
       </c>
       <c r="B96" s="2" t="n">
-        <v>45662.39861111111</v>
+        <v>45663.41805555556</v>
       </c>
       <c r="C96" s="2" t="n">
-        <v>45681.5152986481</v>
+        <v>45687.38881641305</v>
       </c>
       <c r="D96" t="n">
-        <v>27528.03</v>
+        <v>34517.9</v>
       </c>
       <c r="E96" t="n">
-        <v>27220.58</v>
+        <v>34414.2</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-94</t>
         </is>
       </c>
       <c r="B97" s="2" t="n">
-        <v>45662.41944444444</v>
+        <v>45663.42083333333</v>
       </c>
       <c r="C97" s="2" t="n">
-        <v>45682.29557146539</v>
+        <v>45687.48434082514</v>
       </c>
       <c r="D97" t="n">
-        <v>28621.62</v>
+        <v>34651.45</v>
       </c>
       <c r="E97" t="n">
-        <v>28592.06</v>
+        <v>34639.36</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-93</t>
         </is>
       </c>
       <c r="B98" s="2" t="n">
-        <v>45662.40555555555</v>
+        <v>45663.41944444444</v>
       </c>
       <c r="C98" s="2" t="n">
-        <v>45682.30482944068</v>
+        <v>45687.48674930184</v>
       </c>
       <c r="D98" t="n">
-        <v>28654.95</v>
+        <v>34656.92</v>
       </c>
       <c r="E98" t="n">
-        <v>27387.42</v>
+        <v>34513.37</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-95</t>
         </is>
       </c>
       <c r="B99" s="2" t="n">
-        <v>45662.42083333333</v>
+        <v>45663.42222222222</v>
       </c>
       <c r="C99" s="2" t="n">
-        <v>45682.36125961172</v>
+        <v>45687.48880251114</v>
       </c>
       <c r="D99" t="n">
-        <v>28714.21</v>
+        <v>34655.88</v>
       </c>
       <c r="E99" t="n">
-        <v>28689.41</v>
+        <v>34641.11</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-96</t>
         </is>
       </c>
       <c r="B100" s="2" t="n">
-        <v>45662.42222222222</v>
+        <v>45663.42361111111</v>
       </c>
       <c r="C100" s="2" t="n">
-        <v>45682.36506481839</v>
+        <v>45687.49325692131</v>
       </c>
       <c r="D100" t="n">
-        <v>28717.69</v>
+        <v>34660.29</v>
       </c>
       <c r="E100" t="n">
-        <v>28688.22</v>
+        <v>34646.32</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-97</t>
         </is>
       </c>
       <c r="B101" s="2" t="n">
-        <v>45662.42361111111</v>
+        <v>45663.425</v>
       </c>
       <c r="C101" s="2" t="n">
-        <v>45682.36950473118</v>
+        <v>45687.49740479338</v>
       </c>
       <c r="D101" t="n">
-        <v>28722.09</v>
+        <v>34664.26</v>
       </c>
       <c r="E101" t="n">
-        <v>28690.55</v>
+        <v>34649.51</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-98</t>
         </is>
       </c>
       <c r="B102" s="2" t="n">
-        <v>45662.40277777778</v>
+        <v>45663.42638888889</v>
       </c>
       <c r="C102" s="2" t="n">
-        <v>45682.37171391879</v>
+        <v>45688.29722112227</v>
       </c>
       <c r="D102" t="n">
-        <v>28755.27</v>
+        <v>35814</v>
       </c>
       <c r="E102" t="n">
-        <v>28515.25</v>
+        <v>34663.57</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-100</t>
         </is>
       </c>
       <c r="B103" s="2" t="n">
-        <v>45662.425</v>
+        <v>45663.42916666667</v>
       </c>
       <c r="C103" s="2" t="n">
-        <v>45682.37232945213</v>
+        <v>45688.35846367258</v>
       </c>
       <c r="D103" t="n">
-        <v>28724.15</v>
+        <v>35898.19</v>
       </c>
       <c r="E103" t="n">
-        <v>28698.87</v>
+        <v>35884.8</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-99</t>
         </is>
       </c>
       <c r="B104" s="2" t="n">
-        <v>45662.42638888889</v>
+        <v>45663.42777777778</v>
       </c>
       <c r="C104" s="2" t="n">
-        <v>45682.37644474079</v>
+        <v>45688.36337761427</v>
       </c>
       <c r="D104" t="n">
-        <v>28728.08</v>
+        <v>35907.26</v>
       </c>
       <c r="E104" t="n">
-        <v>28700.18</v>
+        <v>35807.88</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-102</t>
         </is>
       </c>
       <c r="B105" s="2" t="n">
-        <v>45662.42777777778</v>
+        <v>45663.43194444444</v>
       </c>
       <c r="C105" s="2" t="n">
-        <v>45682.3806963802</v>
+        <v>45688.45307110677</v>
       </c>
       <c r="D105" t="n">
-        <v>28732.2</v>
+        <v>36030.42</v>
       </c>
       <c r="E105" t="n">
-        <v>28704.42</v>
+        <v>36015.54</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-101</t>
         </is>
       </c>
       <c r="B106" s="2" t="n">
-        <v>45662.42916666667</v>
+        <v>45663.43055555555</v>
       </c>
       <c r="C106" s="2" t="n">
-        <v>45682.38506751259</v>
+        <v>45688.45416635378</v>
       </c>
       <c r="D106" t="n">
-        <v>28736.5</v>
+        <v>36034</v>
       </c>
       <c r="E106" t="n">
-        <v>28709.36</v>
+        <v>35895.52</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-104</t>
         </is>
       </c>
       <c r="B107" s="2" t="n">
-        <v>45662.43055555555</v>
+        <v>45663.43472222222</v>
       </c>
       <c r="C107" s="2" t="n">
-        <v>45682.38970902534</v>
+        <v>45688.45672892279</v>
       </c>
       <c r="D107" t="n">
-        <v>28741.18</v>
+        <v>36031.69</v>
       </c>
       <c r="E107" t="n">
-        <v>28712.76</v>
+        <v>36019.86</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-105</t>
         </is>
       </c>
       <c r="B108" s="2" t="n">
-        <v>45662.43194444444</v>
+        <v>45663.43611111111</v>
       </c>
       <c r="C108" s="2" t="n">
-        <v>45682.39383160766</v>
+        <v>45688.46138404446</v>
       </c>
       <c r="D108" t="n">
-        <v>28745.12</v>
+        <v>36036.39</v>
       </c>
       <c r="E108" t="n">
-        <v>28715.49</v>
+        <v>36020.27</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-107</t>
         </is>
       </c>
       <c r="B109" s="2" t="n">
-        <v>45662.43333333333</v>
+        <v>45663.43888888889</v>
       </c>
       <c r="C109" s="2" t="n">
-        <v>45682.39839205483</v>
+        <v>45691.29459032765</v>
       </c>
       <c r="D109" t="n">
-        <v>28749.68</v>
+        <v>40112.21</v>
       </c>
       <c r="E109" t="n">
-        <v>28721.07</v>
+        <v>40098.89</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-106</t>
         </is>
       </c>
       <c r="B110" s="2" t="n">
-        <v>45662.43611111111</v>
+        <v>45663.4375</v>
       </c>
       <c r="C110" s="2" t="n">
-        <v>45682.40189128138</v>
+        <v>45691.29700716993</v>
       </c>
       <c r="D110" t="n">
-        <v>28750.72</v>
+        <v>40117.69</v>
       </c>
       <c r="E110" t="n">
-        <v>28722.48</v>
+        <v>36032.87</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-108</t>
         </is>
       </c>
       <c r="B111" s="2" t="n">
-        <v>45662.43472222222</v>
+        <v>45663.44027777778</v>
       </c>
       <c r="C111" s="2" t="n">
-        <v>45682.50878649591</v>
+        <v>45691.29916808461</v>
       </c>
       <c r="D111" t="n">
-        <v>28906.65</v>
+        <v>40116.8</v>
       </c>
       <c r="E111" t="n">
-        <v>27638.83</v>
+        <v>40102.64</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-109</t>
         </is>
       </c>
       <c r="B112" s="2" t="n">
-        <v>45662.44027777778</v>
+        <v>45663.44166666667</v>
       </c>
       <c r="C112" s="2" t="n">
-        <v>45683.29476731822</v>
+        <v>45691.30371936662</v>
       </c>
       <c r="D112" t="n">
-        <v>30030.46</v>
+        <v>40121.36</v>
       </c>
       <c r="E112" t="n">
-        <v>30006.79</v>
+        <v>40107.81</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-110</t>
         </is>
       </c>
       <c r="B113" s="2" t="n">
-        <v>45662.44305555556</v>
+        <v>45663.44305555556</v>
       </c>
       <c r="C113" s="2" t="n">
-        <v>45683.298002282</v>
+        <v>45691.30724517736</v>
       </c>
       <c r="D113" t="n">
-        <v>30031.12</v>
+        <v>40124.43</v>
       </c>
       <c r="E113" t="n">
-        <v>30004.98</v>
+        <v>40112.71</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Token-111</t>
         </is>
       </c>
       <c r="B114" s="2" t="n">
-        <v>45662.44444444445</v>
+        <v>45663.44444444445</v>
       </c>
       <c r="C114" s="2" t="n">
-        <v>45683.3022160192</v>
+        <v>45691.31132651552</v>
       </c>
       <c r="D114" t="n">
-        <v>30035.19</v>
+        <v>40128.31</v>
       </c>
       <c r="E114" t="n">
-        <v>30008.65</v>
+        <v>40113.93</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B115" s="2" t="n">
-        <v>45662.44583333333</v>
-      </c>
-      <c r="C115" s="2" t="n">
-        <v>45683.30569821764</v>
-      </c>
-      <c r="D115" t="n">
-        <v>30038.21</v>
-      </c>
-      <c r="E115" t="n">
-        <v>30012.82</v>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B116" s="2" t="n">
-        <v>45662.4375</v>
-      </c>
-      <c r="C116" s="2" t="n">
-        <v>45683.30742214988</v>
-      </c>
-      <c r="D116" t="n">
-        <v>30052.69</v>
-      </c>
-      <c r="E116" t="n">
-        <v>27785.09</v>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B117" s="2" t="n">
-        <v>45662.44861111111</v>
-      </c>
-      <c r="C117" s="2" t="n">
-        <v>45683.30945422715</v>
-      </c>
-      <c r="D117" t="n">
-        <v>30039.61</v>
-      </c>
-      <c r="E117" t="n">
-        <v>30014.03</v>
-      </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B118" s="2" t="n">
-        <v>45662.45277777778</v>
-      </c>
-      <c r="C118" s="2" t="n">
-        <v>45683.31297951594</v>
-      </c>
-      <c r="D118" t="n">
-        <v>30038.69</v>
-      </c>
-      <c r="E118" t="n">
-        <v>30011.46</v>
-      </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B119" s="2" t="n">
-        <v>45662.45416666667</v>
-      </c>
-      <c r="C119" s="2" t="n">
-        <v>45683.3914549181</v>
-      </c>
-      <c r="D119" t="n">
-        <v>30149.7</v>
-      </c>
-      <c r="E119" t="n">
-        <v>30121.08</v>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B120" s="2" t="n">
-        <v>45662.45555555556</v>
-      </c>
-      <c r="C120" s="2" t="n">
-        <v>45683.39545692968</v>
-      </c>
-      <c r="D120" t="n">
-        <v>30153.46</v>
-      </c>
-      <c r="E120" t="n">
-        <v>30129.32</v>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B121" s="2" t="n">
-        <v>45662.44166666667</v>
-      </c>
-      <c r="C121" s="2" t="n">
-        <v>45683.40281377276</v>
-      </c>
-      <c r="D121" t="n">
-        <v>30184.05</v>
-      </c>
-      <c r="E121" t="n">
-        <v>29954.72</v>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B122" s="2" t="n">
-        <v>45662.44722222222</v>
-      </c>
-      <c r="C122" s="2" t="n">
-        <v>45683.48528964628</v>
-      </c>
-      <c r="D122" t="n">
-        <v>30294.82</v>
-      </c>
-      <c r="E122" t="n">
-        <v>30057.57</v>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B123" s="2" t="n">
-        <v>45662.43888888889</v>
-      </c>
-      <c r="C123" s="2" t="n">
-        <v>45683.53375720033</v>
-      </c>
-      <c r="D123" t="n">
-        <v>30376.61</v>
-      </c>
-      <c r="E123" t="n">
-        <v>29038.09</v>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B124" s="2" t="n">
-        <v>45662.45138888889</v>
-      </c>
-      <c r="C124" s="2" t="n">
-        <v>45684.30524191434</v>
-      </c>
-      <c r="D124" t="n">
-        <v>31469.55</v>
-      </c>
-      <c r="E124" t="n">
-        <v>30217.91</v>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B125" s="2" t="n">
-        <v>45662.45</v>
-      </c>
-      <c r="C125" s="2" t="n">
-        <v>45684.40300360583</v>
-      </c>
-      <c r="D125" t="n">
-        <v>31612.33</v>
-      </c>
-      <c r="E125" t="n">
-        <v>31276.63</v>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Work with REO RPO to Correct (5.5.13.3) -&gt; Create Journal Entries? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Create/Post Journal Entries (5.5.13.4) -&gt; Unknown</t>
+          <t>Monthly -&gt; Monthly -&gt; Review AM using Asset Change Tracker (5.5.13.1) -&gt; Complete /Accurate? -&gt; Note Accuracy in Asset Change Tracker (5.5.13.2) -&gt; Unknown</t>
         </is>
       </c>
     </row>
@@ -4082,7 +3818,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>124</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4">
@@ -4092,7 +3828,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>96.77</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -4102,7 +3838,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10.36</v>
+        <v>22875.19</v>
       </c>
     </row>
     <row r="6">
@@ -4112,7 +3848,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11.85</v>
+        <v>35881.35</v>
       </c>
     </row>
     <row r="7">
@@ -4122,7 +3858,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4.46</v>
+        <v>22717.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>